<commit_message>
Invoice Batch Lauf und Feintuning Invoice Template
</commit_message>
<xml_diff>
--- a/templates/time_sheet_template.xlsx
+++ b/templates/time_sheet_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\stephan\projects\wegpiraten\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C394E91-D9BC-4C48-AFCD-38C97B13D136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C1F056C-8FB0-4F1D-A0C4-E574D87E05C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="9r/TxM3zBcSjnJTI/hP9y4R5VkDU9X45pyxBQ1SRhdgGa0G4N9+kmOzqUscJS/8FfSdUOZhKQAU6CU1O1OaWPA==" workbookSaltValue="Ey8SgEponXL1upYzdwO0ww==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="6390" windowWidth="38640" windowHeight="21120" tabRatio="709" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t xml:space="preserve">        </t>
   </si>
@@ -67,16 +67,10 @@
     <t>Fahrtzeit</t>
   </si>
   <si>
-    <t>km</t>
-  </si>
-  <si>
     <t>Direkter Fallkontakt</t>
   </si>
   <si>
     <t>Indirekte Fallbearbeitung</t>
-  </si>
-  <si>
-    <t>Stunden</t>
   </si>
   <si>
     <t xml:space="preserve">Notizen           </t>
@@ -96,15 +90,19 @@
   <si>
     <t>Leistungstyp:</t>
   </si>
+  <si>
+    <t>Summe Zeit</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="0.00;\-0.00;;"/>
-    <numFmt numFmtId="165" formatCode="_ &quot;Fr.&quot;\ * #,##0.00_ ;_ &quot;Fr.&quot;\ * \-#,##0.00_ ;_ &quot;Fr.&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="166" formatCode="[$-407]mmmm\ yy;@"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="_ &quot;Fr.&quot;\ * #,##0.00_ ;_ &quot;Fr.&quot;\ * \-#,##0.00_ ;_ &quot;Fr.&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="[$-407]mmmm\ yy;@"/>
+    <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
+    <numFmt numFmtId="167" formatCode="[h]&quot;h&quot;mm&quot;m&quot;"/>
   </numFmts>
   <fonts count="16" x14ac:knownFonts="1">
     <font>
@@ -227,7 +225,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -321,15 +319,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -338,28 +327,6 @@
         <color indexed="64"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -400,10 +367,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="14"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="14"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="11"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="11"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="20" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
@@ -413,10 +380,6 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -429,15 +392,11 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -448,7 +407,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -476,10 +435,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="17" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -487,9 +443,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -501,49 +454,69 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -557,20 +530,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" readingOrder="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -581,7 +544,12 @@
     <cellStyle name="Eingabe" xfId="1" builtinId="20"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="19">
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -600,202 +568,6 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.00;\-0.00;;"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.00;\-0.00;;"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.00;\-0.00;;"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.00;\-0.00;;"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.00;\-0.00;;"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -835,6 +607,36 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <strike val="0"/>
         <condense val="0"/>
         <extend val="0"/>
@@ -847,7 +649,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="164" formatCode="0.00;\-0.00;;"/>
+      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
       <fill>
         <patternFill>
           <fgColor indexed="64"/>
@@ -870,6 +672,36 @@
         </bottom>
       </border>
       <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -884,7 +716,7 @@
         <name val="Calibri"/>
         <family val="2"/>
       </font>
-      <numFmt numFmtId="164" formatCode="0.00;\-0.00;;"/>
+      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
       <fill>
         <patternFill>
           <fgColor indexed="64"/>
@@ -907,6 +739,36 @@
         </bottom>
       </border>
       <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -921,7 +783,7 @@
         <name val="Calibri"/>
         <family val="2"/>
       </font>
-      <numFmt numFmtId="164" formatCode="0.00;\-0.00;;"/>
+      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
       <fill>
         <patternFill>
           <fgColor indexed="64"/>
@@ -944,6 +806,36 @@
         </bottom>
       </border>
       <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -958,7 +850,7 @@
         <name val="Calibri"/>
         <family val="2"/>
       </font>
-      <numFmt numFmtId="164" formatCode="0.00;\-0.00;;"/>
+      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
       <fill>
         <patternFill>
           <fgColor indexed="64"/>
@@ -984,40 +876,30 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
+        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="10"/>
         <color auto="1"/>
         <name val="Calibri"/>
         <family val="2"/>
+        <scheme val="none"/>
       </font>
-      <numFmt numFmtId="164" formatCode="0.00;\-0.00;;"/>
-      <fill>
-        <patternFill>
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <top/>
+        <bottom/>
       </border>
-      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1055,6 +937,25 @@
         </bottom>
       </border>
       <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1250,14 +1151,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>2904292</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>4732937</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>4732919</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>74792</xdr:rowOff>
     </xdr:to>
@@ -1299,19 +1200,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A10:H29" totalsRowCount="1" headerRowDxfId="19" dataDxfId="18" totalsRowDxfId="16" tableBorderDxfId="17">
-  <autoFilter ref="A10:H28" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Uhrzeit" dataDxfId="15" totalsRowDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Datum" totalsRowLabel="Insgesamt" dataDxfId="14" totalsRowDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Fahrtzeit" totalsRowFunction="sum" dataDxfId="13" totalsRowDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="km" totalsRowFunction="min" dataDxfId="12" totalsRowDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Direkter Fallkontakt" totalsRowFunction="sum" dataDxfId="11" totalsRowDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Indirekte Fallbearbeitung" totalsRowFunction="sum" dataDxfId="10" totalsRowDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Stunden" totalsRowFunction="sum" dataDxfId="9" totalsRowDxfId="1">
-      <calculatedColumnFormula>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</calculatedColumnFormula>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A10:G29" totalsRowCount="1" headerRowDxfId="18" dataDxfId="17" totalsRowDxfId="15" tableBorderDxfId="16">
+  <autoFilter ref="A10:G28" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Uhrzeit" dataDxfId="14" totalsRowDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Datum" totalsRowLabel="Insgesamt" dataDxfId="12" totalsRowDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Fahrtzeit" totalsRowFunction="custom" dataDxfId="10" totalsRowDxfId="9">
+      <totalsRowFormula>ROUNDUP(SUBTOTAL(109,Tabelle1[Fahrtzeit])/5,0)*5</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Notizen           " dataDxfId="8" totalsRowDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Direkter Fallkontakt" totalsRowFunction="custom" dataDxfId="8" totalsRowDxfId="7">
+      <totalsRowFormula>ROUNDUP(SUBTOTAL(109,Tabelle1[Direkter Fallkontakt])/5,0)*5</totalsRowFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Indirekte Fallbearbeitung" totalsRowFunction="custom" dataDxfId="6" totalsRowDxfId="5">
+      <totalsRowFormula>ROUNDUP(SUBTOTAL(109,Tabelle1[Indirekte Fallbearbeitung])/5,0)*5</totalsRowFormula>
+    </tableColumn>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Summe Zeit" totalsRowFunction="sum" dataDxfId="4" totalsRowDxfId="3">
+      <calculatedColumnFormula>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Notizen           " dataDxfId="2" totalsRowDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1667,453 +1573,413 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A3:H34"/>
+  <dimension ref="A3:G33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.23046875" defaultRowHeight="12.9" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.23046875" style="10" customWidth="1"/>
-    <col min="2" max="2" width="10.23046875" style="11" customWidth="1"/>
-    <col min="3" max="3" width="8.23046875" style="12" customWidth="1"/>
-    <col min="4" max="4" width="8.15234375" style="12" customWidth="1"/>
-    <col min="5" max="5" width="12.15234375" style="12" customWidth="1"/>
-    <col min="6" max="6" width="13.84375" style="13" customWidth="1"/>
-    <col min="7" max="7" width="8.61328125" style="12" customWidth="1"/>
-    <col min="8" max="8" width="71.84375" style="14" customWidth="1"/>
-    <col min="9" max="16384" width="11.23046875" style="15"/>
+    <col min="1" max="1" width="11.84375" style="8" customWidth="1"/>
+    <col min="2" max="2" width="11.3046875" style="9" customWidth="1"/>
+    <col min="3" max="3" width="9.3046875" style="10" customWidth="1"/>
+    <col min="4" max="4" width="12.921875" style="10" customWidth="1"/>
+    <col min="5" max="5" width="13.84375" style="11" customWidth="1"/>
+    <col min="6" max="6" width="8.61328125" style="10" customWidth="1"/>
+    <col min="7" max="7" width="71.84375" style="12" customWidth="1"/>
+    <col min="8" max="16384" width="11.23046875" style="13"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A3" s="19" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="20" t="s">
+    <row r="3" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A3" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="18" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="57" t="s">
+    <row r="5" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="55" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="56"/>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="22" t="s">
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="23"/>
-    </row>
-    <row r="6" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="52" t="s">
+      <c r="F5" s="21"/>
+    </row>
+    <row r="6" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="51"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="27"/>
-    </row>
-    <row r="7" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="52" t="s">
+      <c r="B6" s="53"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="24"/>
+    </row>
+    <row r="7" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="54" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="51"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" s="27"/>
-    </row>
-    <row r="8" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="62" t="s">
+      <c r="B7" s="53"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="24"/>
+    </row>
+    <row r="8" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="58" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="51"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="27" t="s">
+      <c r="B8" s="53"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="G8" s="27"/>
-    </row>
-    <row r="9" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="30"/>
-      <c r="B9" s="31"/>
-      <c r="C9" s="32"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="33"/>
-      <c r="G9" s="32"/>
-    </row>
-    <row r="10" spans="1:8" ht="24.55" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="34" t="s">
+      <c r="F8" s="24"/>
+    </row>
+    <row r="9" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="26"/>
+      <c r="B9" s="27"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="28"/>
+    </row>
+    <row r="10" spans="1:7" ht="24.55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="35" t="s">
+      <c r="B10" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="34" t="s">
+      <c r="C10" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="34" t="s">
+      <c r="D10" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="34" t="s">
+      <c r="E10" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="F10" s="36" t="s">
+      <c r="F10" s="33" t="s">
+        <v>19</v>
+      </c>
+      <c r="G10" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="37" t="s">
-        <v>14</v>
-      </c>
-      <c r="H10" s="34" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="18"/>
+    </row>
+    <row r="11" spans="1:7" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="16"/>
       <c r="B11" s="2"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="38">
-        <f>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</f>
-        <v>0</v>
-      </c>
-      <c r="H11" s="8"/>
-    </row>
-    <row r="12" spans="1:8" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="41">
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="6"/>
+    </row>
+    <row r="12" spans="1:7" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1"/>
       <c r="B12" s="2"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="38">
-        <f>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</f>
-        <v>0</v>
-      </c>
-      <c r="H12" s="8"/>
-    </row>
-    <row r="13" spans="1:8" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C12" s="40"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="40"/>
+      <c r="F12" s="41">
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="6"/>
+    </row>
+    <row r="13" spans="1:7" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
       <c r="B13" s="2"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="38">
-        <f>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</f>
-        <v>0</v>
-      </c>
-      <c r="H13" s="8"/>
-    </row>
-    <row r="14" spans="1:8" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C13" s="40"/>
+      <c r="D13" s="40"/>
+      <c r="E13" s="40"/>
+      <c r="F13" s="41">
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="6"/>
+    </row>
+    <row r="14" spans="1:7" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
       <c r="B14" s="2"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="38">
-        <f>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</f>
-        <v>0</v>
-      </c>
-      <c r="H14" s="8"/>
-    </row>
-    <row r="15" spans="1:8" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C14" s="40"/>
+      <c r="D14" s="40"/>
+      <c r="E14" s="40"/>
+      <c r="F14" s="41">
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="6"/>
+    </row>
+    <row r="15" spans="1:7" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
       <c r="B15" s="2"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="38">
-        <f>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="8"/>
-    </row>
-    <row r="16" spans="1:8" s="16" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="41">
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <v>0</v>
+      </c>
+      <c r="G15" s="6"/>
+    </row>
+    <row r="16" spans="1:7" s="14" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="1"/>
       <c r="B16" s="2"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="38">
-        <f>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</f>
-        <v>0</v>
-      </c>
-      <c r="H16" s="8"/>
-    </row>
-    <row r="17" spans="1:8" s="17" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C16" s="40"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="40"/>
+      <c r="F16" s="41">
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <v>0</v>
+      </c>
+      <c r="G16" s="6"/>
+    </row>
+    <row r="17" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="1"/>
       <c r="B17" s="2"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="38">
-        <f>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</f>
-        <v>0</v>
-      </c>
-      <c r="H17" s="8"/>
-    </row>
-    <row r="18" spans="1:8" s="17" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="4"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="40"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="41">
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <v>0</v>
+      </c>
+      <c r="G17" s="6"/>
+    </row>
+    <row r="18" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A18" s="3"/>
       <c r="B18" s="2"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="38">
-        <f>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</f>
-        <v>0</v>
-      </c>
-      <c r="H18" s="8"/>
-    </row>
-    <row r="19" spans="1:8" s="17" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="4"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="40"/>
+      <c r="F18" s="41">
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <v>0</v>
+      </c>
+      <c r="G18" s="6"/>
+    </row>
+    <row r="19" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="3"/>
       <c r="B19" s="2"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="38">
-        <f>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</f>
-        <v>0</v>
-      </c>
-      <c r="H19" s="8"/>
-    </row>
-    <row r="20" spans="1:8" s="17" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="4"/>
+      <c r="C19" s="40"/>
+      <c r="D19" s="40"/>
+      <c r="E19" s="40"/>
+      <c r="F19" s="41">
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <v>0</v>
+      </c>
+      <c r="G19" s="6"/>
+    </row>
+    <row r="20" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A20" s="3"/>
       <c r="B20" s="2"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="38">
-        <f>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</f>
-        <v>0</v>
-      </c>
-      <c r="H20" s="8"/>
-    </row>
-    <row r="21" spans="1:8" s="17" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="4"/>
+      <c r="C20" s="40"/>
+      <c r="D20" s="40"/>
+      <c r="E20" s="40"/>
+      <c r="F20" s="41">
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <v>0</v>
+      </c>
+      <c r="G20" s="6"/>
+    </row>
+    <row r="21" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A21" s="3"/>
       <c r="B21" s="2"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="38">
-        <f>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</f>
-        <v>0</v>
-      </c>
-      <c r="H21" s="8"/>
-    </row>
-    <row r="22" spans="1:8" s="17" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="4"/>
+      <c r="C21" s="40"/>
+      <c r="D21" s="40"/>
+      <c r="E21" s="40"/>
+      <c r="F21" s="41">
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="6"/>
+    </row>
+    <row r="22" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A22" s="3"/>
       <c r="B22" s="2"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="38">
-        <f>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</f>
-        <v>0</v>
-      </c>
-      <c r="H22" s="8"/>
-    </row>
-    <row r="23" spans="1:8" s="17" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="4"/>
+      <c r="C22" s="40"/>
+      <c r="D22" s="40"/>
+      <c r="E22" s="40"/>
+      <c r="F22" s="41">
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <v>0</v>
+      </c>
+      <c r="G22" s="6"/>
+    </row>
+    <row r="23" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A23" s="3"/>
       <c r="B23" s="2"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="38">
-        <f>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</f>
-        <v>0</v>
-      </c>
-      <c r="H23" s="8"/>
-    </row>
-    <row r="24" spans="1:8" s="17" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A24" s="4"/>
+      <c r="C23" s="40"/>
+      <c r="D23" s="40"/>
+      <c r="E23" s="40"/>
+      <c r="F23" s="41">
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <v>0</v>
+      </c>
+      <c r="G23" s="6"/>
+    </row>
+    <row r="24" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A24" s="3"/>
       <c r="B24" s="2"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="38">
-        <f>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</f>
-        <v>0</v>
-      </c>
-      <c r="H24" s="8"/>
-    </row>
-    <row r="25" spans="1:8" s="17" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="4"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="40"/>
+      <c r="E24" s="40"/>
+      <c r="F24" s="41">
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <v>0</v>
+      </c>
+      <c r="G24" s="6"/>
+    </row>
+    <row r="25" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A25" s="3"/>
       <c r="B25" s="2"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
-      <c r="G25" s="38">
-        <f>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</f>
-        <v>0</v>
-      </c>
-      <c r="H25" s="8"/>
-    </row>
-    <row r="26" spans="1:8" s="17" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A26" s="4"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="40"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="41">
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="6"/>
+    </row>
+    <row r="26" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A26" s="3"/>
       <c r="B26" s="2"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="38">
-        <f>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="8"/>
-    </row>
-    <row r="27" spans="1:8" s="17" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="4"/>
+      <c r="C26" s="40"/>
+      <c r="D26" s="40"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="41">
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="6"/>
+    </row>
+    <row r="27" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A27" s="3"/>
       <c r="B27" s="2"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="38">
-        <f>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</f>
-        <v>0</v>
-      </c>
-      <c r="H27" s="8"/>
-    </row>
-    <row r="28" spans="1:8" s="17" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A28" s="5"/>
-      <c r="B28" s="6"/>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="39">
-        <f>SUM(Tabelle1[[#This Row],[Fahrtzeit]],Tabelle1[[#This Row],[Direkter Fallkontakt]],Tabelle1[[#This Row],[Indirekte Fallbearbeitung]])</f>
-        <v>0</v>
-      </c>
-      <c r="H28" s="9"/>
-    </row>
-    <row r="29" spans="1:8" s="17" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="40"/>
-      <c r="B29" s="41" t="s">
+      <c r="C27" s="40"/>
+      <c r="D27" s="40"/>
+      <c r="E27" s="40"/>
+      <c r="F27" s="41">
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <v>0</v>
+      </c>
+      <c r="G27" s="6"/>
+    </row>
+    <row r="28" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A28" s="4"/>
+      <c r="B28" s="5"/>
+      <c r="C28" s="42"/>
+      <c r="D28" s="42"/>
+      <c r="E28" s="42"/>
+      <c r="F28" s="43">
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <v>0</v>
+      </c>
+      <c r="G28" s="7"/>
+    </row>
+    <row r="29" spans="1:7" s="15" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A29" s="34"/>
+      <c r="B29" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="C29" s="44">
+        <f>ROUNDUP(SUBTOTAL(109,Tabelle1[Fahrtzeit])/5,0)*5</f>
+        <v>0</v>
+      </c>
+      <c r="D29" s="44">
+        <f>ROUNDUP(SUBTOTAL(109,Tabelle1[Direkter Fallkontakt])/5,0)*5</f>
+        <v>0</v>
+      </c>
+      <c r="E29" s="44">
+        <f>ROUNDUP(SUBTOTAL(109,Tabelle1[Indirekte Fallbearbeitung])/5,0)*5</f>
+        <v>0</v>
+      </c>
+      <c r="F29" s="45">
+        <f>SUBTOTAL(109,Tabelle1[Summe Zeit])</f>
+        <v>0</v>
+      </c>
+      <c r="G29" s="36"/>
+    </row>
+    <row r="30" spans="1:7" s="15" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A30" s="37"/>
+      <c r="B30" s="9"/>
+      <c r="C30" s="38"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="38"/>
+      <c r="F30" s="39"/>
+      <c r="G30" s="12"/>
+    </row>
+    <row r="31" spans="1:7" s="15" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A31" s="50" t="s">
+        <v>15</v>
+      </c>
+      <c r="B31" s="51"/>
+      <c r="C31" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="C29" s="42">
-        <f>SUBTOTAL(109,Tabelle1[Fahrtzeit])</f>
-        <v>0</v>
-      </c>
-      <c r="D29" s="42">
-        <f>SUBTOTAL(105,Tabelle1[km])</f>
-        <v>0</v>
-      </c>
-      <c r="E29" s="42">
-        <f>SUBTOTAL(109,Tabelle1[Direkter Fallkontakt])</f>
-        <v>0</v>
-      </c>
-      <c r="F29" s="42">
-        <f>SUBTOTAL(109,Tabelle1[Indirekte Fallbearbeitung])</f>
-        <v>0</v>
-      </c>
-      <c r="G29" s="43">
-        <f>SUBTOTAL(109,Tabelle1[Stunden])</f>
-        <v>0</v>
-      </c>
-      <c r="H29" s="44"/>
-    </row>
-    <row r="30" spans="1:8" s="17" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="45"/>
-      <c r="B30" s="11"/>
-      <c r="C30" s="46"/>
-      <c r="D30" s="46"/>
-      <c r="E30" s="46"/>
-      <c r="F30" s="46"/>
-      <c r="G30" s="47"/>
-      <c r="H30" s="14"/>
-    </row>
-    <row r="31" spans="1:8" s="17" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="48" t="s">
+      <c r="D31" s="53"/>
+      <c r="E31" s="51"/>
+      <c r="F31" s="57" t="s">
         <v>17</v>
       </c>
-      <c r="B31" s="49"/>
-      <c r="C31" s="50" t="s">
-        <v>18</v>
-      </c>
-      <c r="D31" s="51"/>
-      <c r="E31" s="51"/>
-      <c r="F31" s="49"/>
-      <c r="G31" s="61" t="s">
-        <v>19</v>
-      </c>
-      <c r="H31" s="49"/>
-    </row>
-    <row r="32" spans="1:8" s="17" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="58">
-        <f>C7</f>
-        <v>0</v>
-      </c>
-      <c r="B32" s="59"/>
-      <c r="C32" s="58">
-        <f>Tabelle1[[#Totals],[Stunden]]</f>
-        <v>0</v>
-      </c>
-      <c r="D32" s="54"/>
-      <c r="E32" s="54"/>
-      <c r="F32" s="59"/>
-      <c r="G32" s="53">
-        <f>C32-A32</f>
-        <v>0</v>
-      </c>
-      <c r="H32" s="54"/>
-    </row>
-    <row r="33" spans="1:8" s="17" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="55"/>
-      <c r="B33" s="60"/>
-      <c r="C33" s="55"/>
-      <c r="D33" s="56"/>
-      <c r="E33" s="56"/>
-      <c r="F33" s="60"/>
-      <c r="G33" s="55"/>
-      <c r="H33" s="56"/>
-    </row>
-    <row r="34" spans="1:8" s="17" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A34" s="15"/>
-      <c r="B34" s="15"/>
-      <c r="C34" s="15"/>
-      <c r="D34" s="15"/>
-      <c r="E34" s="15"/>
-      <c r="F34" s="15"/>
-      <c r="G34" s="15"/>
-      <c r="H34" s="15"/>
+      <c r="G31" s="51"/>
+    </row>
+    <row r="32" spans="1:7" s="15" customFormat="1" ht="31.3" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A32" s="47">
+        <f>$C$7*60/1440</f>
+        <v>0</v>
+      </c>
+      <c r="B32" s="48"/>
+      <c r="C32" s="47">
+        <f>Tabelle1[[#Totals],[Summe Zeit]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="D32" s="48"/>
+      <c r="E32" s="49"/>
+      <c r="F32" s="47">
+        <f>ABS(C32-A32)</f>
+        <v>0</v>
+      </c>
+      <c r="G32" s="48"/>
+    </row>
+    <row r="33" spans="1:7" s="15" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A33" s="13"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="13"/>
+      <c r="F33" s="13"/>
+      <c r="G33" s="13"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="RVtKP3YgTW2tCZgRJr5UlEEBh2ANPkAni/YaBDcHzSEvma/7gUX8Z90TxtN8wBTzeaw5RZKcfIiD1a+VM6pgEQ==" saltValue="bJ9myUyMUPCmTECEa79wAw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="N7aNfOtwNi0srLuSnj2/88MC+rJLPT7Xak/aucOtmo2W0fiZxmhCR7W1T7ri4SBvoo/Cb25MRp1zrEzp09hfCg==" saltValue="HhTLFLDcWytS3cHgkFsMGQ==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="10">
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="C31:F31"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="G32:H33"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A32:B33"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="C32:F33"/>
+    <mergeCell ref="F31:G31"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="C31:E31"/>
   </mergeCells>
+  <conditionalFormatting sqref="F32:G32">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>$A32&lt;$C32</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
   <headerFooter differentFirst="1">
@@ -2125,9 +1991,9 @@
 Familienbegleitung&amp;K00+000A</oddFooter>
     <firstHeader>&amp;LV5.0 autom
 &amp;RC3 - Vertraulich</firstHeader>
-    <firstFooter>&amp;L&amp;7 Wegpiraten GmbH
-Alpenstrasse 2
-3800 Interlaken&amp;C&amp;7 Tel: 076 790 67 56
+    <firstFooter>&amp;L&amp;7Wegpiraten GmbH
+Hauptstraße 47
+3800 Unterlakjen&amp;C&amp;7 Tel: 076 790 67 56
              E-Mail: info@wegpiraten.ch
  www.wegpiraten.ch&amp;R&amp;7 &amp;K000000Sozialpädagogische        &amp;K00+000A
 Familienbegleitung          F</firstFooter>

</xml_diff>

<commit_message>
Bugfixes: Font-Fallback, Spaltennamen Rechnungsübersicht, FK-Feldnamen Timesheets
- invoice_factory: Font-Fallback-Kette (Calibri via WSL, Liberation Sans, DejaVu)
- document_utils: Spalten umbenannt (Soll→Max, Leistungszeit entfernt), bedingte
  Formatierung hellrot wenn Ist > Max für alle Max/Ist-Paare
- batch_import_timesheets: Zeiten nicht mehr mit 60 multiplizieren (bereits Minuten)
- time_sheet_factory/batch_processor: FK-Feldnamen auf allowed_travel_time,
  allowed_direct_effort, allowed_indirect_effort korrigiert

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/time_sheet_template.xlsx
+++ b/templates/time_sheet_template.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\stephan\projects\wegpiraten\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Debian\home\stephan\projects\wegpiraten\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C1F056C-8FB0-4F1D-A0C4-E574D87E05C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EF925C2-3F75-49C0-8F0B-38C1713889AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="9r/TxM3zBcSjnJTI/hP9y4R5VkDU9X45pyxBQ1SRhdgGa0G4N9+kmOzqUscJS/8FfSdUOZhKQAU6CU1O1OaWPA==" workbookSaltValue="Ey8SgEponXL1upYzdwO0ww==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="6390" windowWidth="38640" windowHeight="21120" tabRatio="709" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="709" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arbeitszeiterfassung" sheetId="1" r:id="rId1"/>
@@ -35,9 +35,6 @@
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t xml:space="preserve">        </t>
-  </si>
-  <si>
-    <t>Arbeitszeiterfassung</t>
   </si>
   <si>
     <t>Mitarbeiter*in:</t>
@@ -92,6 +89,9 @@
   </si>
   <si>
     <t>Summe Zeit</t>
+  </si>
+  <si>
+    <t>Zeiterfassung</t>
   </si>
 </sst>
 </file>
@@ -510,26 +510,10 @@
     <xf numFmtId="1" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" readingOrder="1"/>
     </xf>
@@ -537,7 +521,23 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Berechnung" xfId="2" builtinId="22"/>
@@ -1574,73 +1574,73 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A3:G33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.23046875" defaultRowHeight="12.9" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.26953125" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.84375" style="8" customWidth="1"/>
-    <col min="2" max="2" width="11.3046875" style="9" customWidth="1"/>
-    <col min="3" max="3" width="9.3046875" style="10" customWidth="1"/>
-    <col min="4" max="4" width="12.921875" style="10" customWidth="1"/>
-    <col min="5" max="5" width="13.84375" style="11" customWidth="1"/>
-    <col min="6" max="6" width="8.61328125" style="10" customWidth="1"/>
-    <col min="7" max="7" width="71.84375" style="12" customWidth="1"/>
-    <col min="8" max="16384" width="11.23046875" style="13"/>
+    <col min="1" max="1" width="11.81640625" style="8" customWidth="1"/>
+    <col min="2" max="2" width="11.26953125" style="9" customWidth="1"/>
+    <col min="3" max="3" width="9.26953125" style="10" customWidth="1"/>
+    <col min="4" max="4" width="12.90625" style="10" customWidth="1"/>
+    <col min="5" max="5" width="13.81640625" style="11" customWidth="1"/>
+    <col min="6" max="6" width="8.6328125" style="10" customWidth="1"/>
+    <col min="7" max="7" width="71.81640625" style="12" customWidth="1"/>
+    <col min="8" max="16384" width="11.26953125" style="13"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="3" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A3" s="17" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="18" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="49" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="55" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="56"/>
+      <c r="B5" s="50"/>
       <c r="C5" s="19"/>
       <c r="D5" s="19"/>
       <c r="E5" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="F5" s="21"/>
+    </row>
+    <row r="6" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="F5" s="21"/>
-    </row>
-    <row r="6" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="54" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="53"/>
+      <c r="B6" s="48"/>
       <c r="C6" s="22"/>
       <c r="D6" s="23"/>
       <c r="E6" s="20"/>
       <c r="F6" s="24"/>
     </row>
-    <row r="7" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="54" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="53"/>
+    <row r="7" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="47" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="48"/>
       <c r="C7" s="46"/>
       <c r="D7" s="25"/>
       <c r="E7" s="21" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F7" s="24"/>
     </row>
-    <row r="8" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="58" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="53"/>
+    <row r="8" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="53" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="48"/>
       <c r="C8" s="23"/>
       <c r="D8" s="23"/>
       <c r="E8" s="24" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F8" s="24"/>
     </row>
-    <row r="9" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="26"/>
       <c r="B9" s="27"/>
       <c r="C9" s="28"/>
@@ -1648,30 +1648,30 @@
       <c r="E9" s="29"/>
       <c r="F9" s="28"/>
     </row>
-    <row r="10" spans="1:7" ht="24.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" ht="24.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="30" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="31" t="s">
+      <c r="C10" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="30" t="s">
+      <c r="D10" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="30" t="s">
+      <c r="E10" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="32" t="s">
+      <c r="F10" s="33" t="s">
+        <v>18</v>
+      </c>
+      <c r="G10" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="F10" s="33" t="s">
-        <v>19</v>
-      </c>
-      <c r="G10" s="30" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:7" ht="14.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="16"/>
       <c r="B11" s="2"/>
       <c r="C11" s="40"/>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="G11" s="6"/>
     </row>
-    <row r="12" spans="1:7" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" ht="14.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="2"/>
       <c r="C12" s="40"/>
@@ -1695,7 +1695,7 @@
       </c>
       <c r="G12" s="6"/>
     </row>
-    <row r="13" spans="1:7" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" ht="14.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="2"/>
       <c r="C13" s="40"/>
@@ -1707,7 +1707,7 @@
       </c>
       <c r="G13" s="6"/>
     </row>
-    <row r="14" spans="1:7" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" ht="14.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="2"/>
       <c r="C14" s="40"/>
@@ -1719,7 +1719,7 @@
       </c>
       <c r="G14" s="6"/>
     </row>
-    <row r="15" spans="1:7" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="14.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="2"/>
       <c r="C15" s="40"/>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="G15" s="6"/>
     </row>
-    <row r="16" spans="1:7" s="14" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" s="14" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
       <c r="B16" s="2"/>
       <c r="C16" s="40"/>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="G16" s="6"/>
     </row>
-    <row r="17" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
       <c r="B17" s="2"/>
       <c r="C17" s="40"/>
@@ -1755,7 +1755,7 @@
       </c>
       <c r="G17" s="6"/>
     </row>
-    <row r="18" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3"/>
       <c r="B18" s="2"/>
       <c r="C18" s="40"/>
@@ -1767,7 +1767,7 @@
       </c>
       <c r="G18" s="6"/>
     </row>
-    <row r="19" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3"/>
       <c r="B19" s="2"/>
       <c r="C19" s="40"/>
@@ -1779,7 +1779,7 @@
       </c>
       <c r="G19" s="6"/>
     </row>
-    <row r="20" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3"/>
       <c r="B20" s="2"/>
       <c r="C20" s="40"/>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="G20" s="6"/>
     </row>
-    <row r="21" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3"/>
       <c r="B21" s="2"/>
       <c r="C21" s="40"/>
@@ -1803,7 +1803,7 @@
       </c>
       <c r="G21" s="6"/>
     </row>
-    <row r="22" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3"/>
       <c r="B22" s="2"/>
       <c r="C22" s="40"/>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="G22" s="6"/>
     </row>
-    <row r="23" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3"/>
       <c r="B23" s="2"/>
       <c r="C23" s="40"/>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="G23" s="6"/>
     </row>
-    <row r="24" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3"/>
       <c r="B24" s="2"/>
       <c r="C24" s="40"/>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="G24" s="6"/>
     </row>
-    <row r="25" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="3"/>
       <c r="B25" s="2"/>
       <c r="C25" s="40"/>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="G25" s="6"/>
     </row>
-    <row r="26" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="3"/>
       <c r="B26" s="2"/>
       <c r="C26" s="40"/>
@@ -1863,7 +1863,7 @@
       </c>
       <c r="G26" s="6"/>
     </row>
-    <row r="27" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="3"/>
       <c r="B27" s="2"/>
       <c r="C27" s="40"/>
@@ -1875,7 +1875,7 @@
       </c>
       <c r="G27" s="6"/>
     </row>
-    <row r="28" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:7" s="15" customFormat="1" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="4"/>
       <c r="B28" s="5"/>
       <c r="C28" s="42"/>
@@ -1887,10 +1887,10 @@
       </c>
       <c r="G28" s="7"/>
     </row>
-    <row r="29" spans="1:7" s="15" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7" s="15" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="34"/>
       <c r="B29" s="35" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C29" s="44">
         <f>ROUNDUP(SUBTOTAL(109,Tabelle1[Fahrtzeit])/5,0)*5</f>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="G29" s="36"/>
     </row>
-    <row r="30" spans="1:7" s="15" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" s="15" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="37"/>
       <c r="B30" s="9"/>
       <c r="C30" s="38"/>
@@ -1919,40 +1919,40 @@
       <c r="F30" s="39"/>
       <c r="G30" s="12"/>
     </row>
-    <row r="31" spans="1:7" s="15" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="50" t="s">
+    <row r="31" spans="1:7" s="15" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="57" t="s">
+        <v>14</v>
+      </c>
+      <c r="B31" s="52"/>
+      <c r="C31" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="51"/>
-      <c r="C31" s="52" t="s">
+      <c r="D31" s="48"/>
+      <c r="E31" s="52"/>
+      <c r="F31" s="51" t="s">
         <v>16</v>
       </c>
-      <c r="D31" s="53"/>
-      <c r="E31" s="51"/>
-      <c r="F31" s="57" t="s">
-        <v>17</v>
-      </c>
-      <c r="G31" s="51"/>
-    </row>
-    <row r="32" spans="1:7" s="15" customFormat="1" ht="31.3" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="47">
+      <c r="G31" s="52"/>
+    </row>
+    <row r="32" spans="1:7" s="15" customFormat="1" ht="31.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="54">
         <f>$C$7*60/1440</f>
         <v>0</v>
       </c>
-      <c r="B32" s="48"/>
-      <c r="C32" s="47">
+      <c r="B32" s="55"/>
+      <c r="C32" s="54">
         <f>Tabelle1[[#Totals],[Summe Zeit]]/1440</f>
         <v>0</v>
       </c>
-      <c r="D32" s="48"/>
-      <c r="E32" s="49"/>
-      <c r="F32" s="47">
+      <c r="D32" s="55"/>
+      <c r="E32" s="56"/>
+      <c r="F32" s="54">
         <f>ABS(C32-A32)</f>
         <v>0</v>
       </c>
-      <c r="G32" s="48"/>
-    </row>
-    <row r="33" spans="1:7" s="15" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="G32" s="55"/>
+    </row>
+    <row r="33" spans="1:7" s="15" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="13"/>
       <c r="B33" s="13"/>
       <c r="C33" s="13"/>
@@ -1962,18 +1962,18 @@
       <c r="G33" s="13"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="N7aNfOtwNi0srLuSnj2/88MC+rJLPT7Xak/aucOtmo2W0fiZxmhCR7W1T7ri4SBvoo/Cb25MRp1zrEzp09hfCg==" saltValue="HhTLFLDcWytS3cHgkFsMGQ==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="O6qruKqfHk6ijjlA3ETq1C3qDDbJJhSnbjV3rD/48lJZ3c/TeOjGQoKObL8cRQmUYXY/MRmRYeYX7wixoWvgHg==" saltValue="adVFvDA7fG289mllICikBQ==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="10">
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="C31:E31"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="F31:G31"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="C31:E31"/>
   </mergeCells>
   <conditionalFormatting sqref="F32:G32">
     <cfRule type="expression" dxfId="0" priority="1">

</xml_diff>

<commit_message>
Bugfix: SPC-Zahlschein zeigt Tenant-Daten (IBAN, Anschrift, Name); Tenant-name-Feld im Import
- SPC/Zahlschein nutzt klientenspezifische Tenant-IBAN und -Anschrift statt globaler Config
- Tenant-Modell um Namensfeld erweitert (YAML, SQL, Context, Factory)
- ALTER TABLE-Migration für bestehende DBs (name-Spalte)
- make timesheets speichert MONTH nicht mehr in .month

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/time_sheet_template.xlsx
+++ b/templates/time_sheet_template.xlsx
@@ -1,126 +1,205 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
-  <workbookProtection lockStructure="1" workbookAlgorithmName="SHA-512" workbookHashValue="9r/TxM3zBcSjnJTI/hP9y4R5VkDU9X45pyxBQ1SRhdgGa0G4N9+kmOzqUscJS/8FfSdUOZhKQAU6CU1O1OaWPA==" workbookSaltValue="Ey8SgEponXL1upYzdwO0ww==" workbookSpinCount="100000"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Debian\home\stephan\projects\wegpiraten\templates\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAF65A4C-E47F-42DA-B25C-0D9DA0A328FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="9r/TxM3zBcSjnJTI/hP9y4R5VkDU9X45pyxBQ1SRhdgGa0G4N9+kmOzqUscJS/8FfSdUOZhKQAU6CU1O1OaWPA==" workbookSaltValue="Ey8SgEponXL1upYzdwO0ww==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" tabRatio="709" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="57480" yWindow="6390" windowWidth="38640" windowHeight="21120" tabRatio="709" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Arbeitszeiterfassung" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Arbeitszeiterfassung" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+  <si>
+    <t xml:space="preserve">        </t>
+  </si>
+  <si>
+    <t>Zeiterfassung</t>
+  </si>
+  <si>
+    <t>Mitarbeiter*in:</t>
+  </si>
+  <si>
+    <t>Ma-Nr.:</t>
+  </si>
+  <si>
+    <t>Monat/Jahr:</t>
+  </si>
+  <si>
+    <t>Max Stunden/Monat:</t>
+  </si>
+  <si>
+    <t>Leistungstyp:</t>
+  </si>
+  <si>
+    <t>Klient*in:</t>
+  </si>
+  <si>
+    <t>Klient-Nr.:</t>
+  </si>
+  <si>
+    <t>Uhrzeit</t>
+  </si>
+  <si>
+    <t>Datum</t>
+  </si>
+  <si>
+    <t>Fahrtzeit</t>
+  </si>
+  <si>
+    <t>Direkter Fallkontakt</t>
+  </si>
+  <si>
+    <t>Indirekte Fallbearbeitung</t>
+  </si>
+  <si>
+    <t>Summe Zeit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notizen           </t>
+  </si>
+  <si>
+    <t>Insgesamt</t>
+  </si>
+  <si>
+    <t>Obergrenze</t>
+  </si>
+  <si>
+    <t>Differenz</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="_ &quot;Fr.&quot;\ * #,##0.00_ ;_ &quot;Fr.&quot;\ * \-#,##0.00_ ;_ &quot;Fr.&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="165" formatCode="[$-407]mmmm\ yy;@"/>
     <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
     <numFmt numFmtId="167" formatCode="[h]&quot;h&quot;mm&quot;m&quot;"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
+      <sz val="10"/>
       <name val="Arial"/>
-      <sz val="10"/>
     </font>
     <font>
+      <sz val="10"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <sz val="10"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="10"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <sz val="10"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="17"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <sz val="17"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="12"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="12"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <sz val="10"/>
     </font>
     <font>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
-      <sz val="10"/>
     </font>
     <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <sz val="11"/>
     </font>
     <font>
+      <b/>
+      <sz val="10"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <sz val="10"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color rgb="FF3F3F76"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color theme="0"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="0"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -136,7 +215,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -275,15 +354,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -291,173 +361,173 @@
     <xf numFmtId="0" fontId="12" fillId="3" borderId="11"/>
   </cellStyleXfs>
   <cellXfs count="56">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="20" fontId="7" fillId="0" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="20" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="8" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="17" fontId="7" fillId="0" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="17" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="4" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="4" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
+    <cellStyle name="Berechnung" xfId="2" builtinId="22"/>
+    <cellStyle name="Eingabe" xfId="1" builtinId="20"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
-    <cellStyle name="Eingabe" xfId="1" builtinId="20"/>
-    <cellStyle name="Berechnung" xfId="2" builtinId="22"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="21">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -484,31 +554,31 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
         <name val="Calibri"/>
         <family val="2"/>
+      </font>
+      <alignment horizontal="left" vertical="bottom"/>
+    </dxf>
+    <dxf>
+      <font>
         <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <condense val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
         <color auto="1"/>
-        <extend val="0"/>
-        <sz val="10"/>
-        <vertAlign val="baseline"/>
-      </font>
-      <alignment horizontal="left" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <font>
         <name val="Calibri"/>
         <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-        <sz val="10"/>
-        <vertAlign val="baseline"/>
       </font>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
@@ -534,17 +604,17 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
         <name val="Calibri"/>
         <family val="2"/>
-        <b val="1"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-        <sz val="10"/>
-        <vertAlign val="baseline"/>
         <scheme val="minor"/>
       </font>
       <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
@@ -562,17 +632,17 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
         <name val="Calibri"/>
         <family val="2"/>
-        <b val="1"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-        <sz val="10"/>
-        <vertAlign val="baseline"/>
         <scheme val="minor"/>
       </font>
       <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
@@ -601,17 +671,17 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
         <name val="Calibri"/>
         <family val="2"/>
-        <b val="1"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-        <sz val="10"/>
-        <vertAlign val="baseline"/>
       </font>
       <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
       <alignment horizontal="center" vertical="center"/>
@@ -628,16 +698,16 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
         <name val="Calibri"/>
         <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-        <sz val="10"/>
-        <vertAlign val="baseline"/>
       </font>
       <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
       <fill>
@@ -665,17 +735,17 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
         <name val="Calibri"/>
         <family val="2"/>
-        <b val="1"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-        <sz val="10"/>
-        <vertAlign val="baseline"/>
       </font>
       <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
       <alignment horizontal="center" vertical="center"/>
@@ -692,16 +762,16 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
         <name val="Calibri"/>
         <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-        <sz val="10"/>
-        <vertAlign val="baseline"/>
       </font>
       <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
       <fill>
@@ -729,17 +799,17 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
         <name val="Calibri"/>
         <family val="2"/>
-        <b val="1"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-        <sz val="10"/>
-        <vertAlign val="baseline"/>
       </font>
       <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
       <alignment horizontal="center" vertical="center"/>
@@ -756,16 +826,16 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
         <name val="Calibri"/>
         <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-        <sz val="10"/>
-        <vertAlign val="baseline"/>
       </font>
       <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
       <fill>
@@ -793,16 +863,16 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
         <name val="Calibri"/>
         <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-        <sz val="10"/>
-        <vertAlign val="baseline"/>
       </font>
       <alignment horizontal="right" vertical="bottom"/>
       <border outline="0">
@@ -816,16 +886,16 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
         <name val="Calibri"/>
         <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-        <sz val="10"/>
-        <vertAlign val="baseline"/>
       </font>
       <numFmt numFmtId="1" formatCode="0"/>
       <fill>
@@ -853,31 +923,31 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
         <name val="Calibri"/>
         <family val="2"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom"/>
+    </dxf>
+    <dxf>
+      <font>
         <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <condense val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
         <color auto="1"/>
-        <extend val="0"/>
-        <sz val="10"/>
-        <vertAlign val="baseline"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <font>
         <name val="Calibri"/>
         <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-        <sz val="10"/>
-        <vertAlign val="baseline"/>
       </font>
       <fill>
         <patternFill>
@@ -921,16 +991,16 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
         <name val="Calibri"/>
         <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-        <sz val="10"/>
-        <vertAlign val="baseline"/>
       </font>
       <fill>
         <patternFill>
@@ -943,17 +1013,17 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
         <name val="Calibri"/>
         <family val="2"/>
-        <b val="1"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color theme="0"/>
-        <extend val="0"/>
-        <sz val="11"/>
-        <vertAlign val="baseline"/>
         <scheme val="minor"/>
       </font>
       <fill>
@@ -974,30 +1044,6 @@
         <bottom/>
       </border>
       <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFCCCC"/>
-          <bgColor rgb="00FFCCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFFF99"/>
-          <bgColor rgb="00FFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00B3FFD9"/>
-          <bgColor rgb="00B3FFD9"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1069,74 +1115,88 @@
       <rgbColor rgb="00424242"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>6</col>
-      <colOff>2904292</colOff>
-      <row>0</row>
-      <rowOff>38100</rowOff>
-    </from>
-    <to>
-      <col>7</col>
-      <colOff>54239</colOff>
-      <row>8</row>
-      <rowOff>74792</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Grafik 1"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>2732842</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>6350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>4562739</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>49392</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Grafik 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="7914442" y="38100"/>
-          <a:ext cx="1830010" cy="1547992"/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7781092" y="6350"/>
+          <a:ext cx="1829897" cy="1528942"/>
         </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
         </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabelle1" displayName="Tabelle1" ref="A10:G29" headerRowCount="1" totalsRowCount="1" headerRowDxfId="20" dataDxfId="19" totalsRowDxfId="17" tableBorderDxfId="18">
-  <autoFilter ref="A10:G28"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A10:G29" totalsRowCount="1" headerRowDxfId="20" dataDxfId="19" totalsRowDxfId="17" tableBorderDxfId="18">
+  <autoFilter ref="A10:G28" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="7">
-    <tableColumn id="1" name="Uhrzeit" dataDxfId="16" totalsRowDxfId="15"/>
-    <tableColumn id="2" name="Datum" totalsRowLabel="Insgesamt" dataDxfId="14" totalsRowDxfId="13"/>
-    <tableColumn id="3" name="Fahrtzeit" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="11">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Uhrzeit" dataDxfId="16" totalsRowDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Datum" totalsRowLabel="Insgesamt" dataDxfId="14" totalsRowDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Fahrtzeit" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="11">
       <totalsRowFormula>ROUNDUP(SUBTOTAL(109,Tabelle1[Fahrtzeit])/5,0)*5</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="5" name="Direkter Fallkontakt" totalsRowFunction="custom" dataDxfId="10" totalsRowDxfId="9">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Direkter Fallkontakt" totalsRowFunction="custom" dataDxfId="10" totalsRowDxfId="9">
       <totalsRowFormula>ROUNDUP(SUBTOTAL(109,Tabelle1[Direkter Fallkontakt])/5,0)*5</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="6" name="Indirekte Fallbearbeitung" totalsRowFunction="custom" dataDxfId="8" totalsRowDxfId="7">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Indirekte Fallbearbeitung" totalsRowFunction="custom" dataDxfId="8" totalsRowDxfId="7">
       <totalsRowFormula>ROUNDUP(SUBTOTAL(109,Tabelle1[Indirekte Fallbearbeitung])/5,0)*5</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="7" name="Summe Zeit" totalsRowFunction="sum" dataDxfId="6" totalsRowDxfId="5">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Summe Zeit" totalsRowFunction="sum" dataDxfId="6" totalsRowDxfId="5">
       <calculatedColumnFormula>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" name="Notizen           " dataDxfId="4" totalsRowDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Notizen           " dataDxfId="4" totalsRowDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1491,438 +1551,396 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A3:G33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.27734375" defaultRowHeight="12.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.26953125" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col width="11.83203125" customWidth="1" style="6" min="1" max="1"/>
-    <col width="11.27734375" customWidth="1" style="7" min="2" max="2"/>
-    <col width="9.27734375" customWidth="1" style="8" min="3" max="3"/>
-    <col width="12.88671875" customWidth="1" style="8" min="4" max="4"/>
-    <col width="13.83203125" customWidth="1" style="9" min="5" max="5"/>
-    <col width="12.83203125" customWidth="1" style="8" min="6" max="6"/>
-    <col width="66.71875" customWidth="1" style="10" min="7" max="7"/>
-    <col width="11.27734375" customWidth="1" style="11" min="8" max="8"/>
-    <col width="11.27734375" customWidth="1" style="11" min="9" max="16384"/>
+    <col min="1" max="1" width="11.81640625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="11.26953125" style="7" customWidth="1"/>
+    <col min="3" max="3" width="9.26953125" style="8" customWidth="1"/>
+    <col min="4" max="4" width="12.90625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="13.81640625" style="9" customWidth="1"/>
+    <col min="6" max="6" width="12.81640625" style="8" customWidth="1"/>
+    <col min="7" max="7" width="66.7265625" style="10" customWidth="1"/>
+    <col min="8" max="16384" width="11.26953125" style="11"/>
   </cols>
   <sheetData>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        </t>
-        </is>
-      </c>
-      <c r="B3" s="16" t="inlineStr">
-        <is>
-          <t>Zeiterfassung</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="14.5" customHeight="1">
-      <c r="A5" s="53" t="inlineStr">
-        <is>
-          <t>Mitarbeiter*in:</t>
-        </is>
-      </c>
-      <c r="B5" s="54" t="n"/>
-      <c r="C5" s="17" t="n"/>
-      <c r="D5" s="17" t="n"/>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>Ma-Nr.:</t>
-        </is>
-      </c>
-      <c r="F5" s="19" t="n"/>
-    </row>
-    <row r="6" ht="14.5" customHeight="1">
-      <c r="A6" s="51" t="inlineStr">
-        <is>
-          <t>Monat/Jahr:</t>
-        </is>
-      </c>
-      <c r="B6" s="52" t="n"/>
-      <c r="C6" s="20" t="n"/>
-      <c r="D6" s="21" t="n"/>
-      <c r="E6" s="18" t="n"/>
-      <c r="F6" s="22" t="n"/>
-    </row>
-    <row r="7" ht="14.5" customHeight="1">
-      <c r="A7" s="51" t="inlineStr">
-        <is>
-          <t>Max Stunden/Monat:</t>
-        </is>
-      </c>
-      <c r="B7" s="52" t="n"/>
-      <c r="C7" s="40" t="n"/>
-      <c r="D7" s="23" t="n"/>
-      <c r="E7" s="19" t="inlineStr">
-        <is>
-          <t>Leistungstyp:</t>
-        </is>
-      </c>
-      <c r="F7" s="22" t="n"/>
-    </row>
-    <row r="8" ht="14.5" customHeight="1">
-      <c r="A8" s="55" t="inlineStr">
-        <is>
-          <t>Klient*in:</t>
-        </is>
-      </c>
-      <c r="B8" s="52" t="n"/>
-      <c r="C8" s="21" t="n"/>
-      <c r="D8" s="21" t="n"/>
-      <c r="E8" s="22" t="inlineStr">
-        <is>
-          <t>Klient-Nr.:</t>
-        </is>
-      </c>
-      <c r="F8" s="22" t="n"/>
-    </row>
-    <row r="9" ht="14.5" customHeight="1">
-      <c r="A9" s="24" t="n"/>
-      <c r="B9" s="25" t="n"/>
-      <c r="C9" s="26" t="n"/>
-      <c r="D9" s="26" t="n"/>
-      <c r="E9" s="27" t="n"/>
-      <c r="F9" s="26" t="n"/>
-    </row>
-    <row r="10" ht="24.55" customHeight="1">
-      <c r="A10" s="28" t="inlineStr">
-        <is>
-          <t>Uhrzeit</t>
-        </is>
-      </c>
-      <c r="B10" s="29" t="inlineStr">
-        <is>
-          <t>Datum</t>
-        </is>
-      </c>
-      <c r="C10" s="28" t="inlineStr">
-        <is>
-          <t>Fahrtzeit</t>
-        </is>
-      </c>
-      <c r="D10" s="28" t="inlineStr">
-        <is>
-          <t>Direkter Fallkontakt</t>
-        </is>
-      </c>
-      <c r="E10" s="30" t="inlineStr">
-        <is>
-          <t>Indirekte Fallbearbeitung</t>
-        </is>
-      </c>
-      <c r="F10" s="31" t="inlineStr">
-        <is>
-          <t>Summe Zeit</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Notizen           </t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="14.2" customHeight="1">
-      <c r="A11" s="14" t="n"/>
-      <c r="B11" s="49" t="n"/>
-      <c r="C11" s="34" t="n"/>
-      <c r="D11" s="34" t="n"/>
-      <c r="E11" s="34" t="n"/>
+    <row r="3" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A3" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="54" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="55"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" s="19"/>
+    </row>
+    <row r="6" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="52"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="22"/>
+    </row>
+    <row r="7" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="53" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="52"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="F7" s="22"/>
+    </row>
+    <row r="8" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="51" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="52"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="22"/>
+    </row>
+    <row r="9" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="24"/>
+      <c r="B9" s="25"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="26"/>
+    </row>
+    <row r="10" spans="1:7" ht="24.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="30" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" s="28" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="14"/>
+      <c r="B11" s="49"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="34"/>
       <c r="F11" s="35">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
-        <v/>
-      </c>
-      <c r="G11" s="4" t="n"/>
-    </row>
-    <row r="12" ht="14.2" customHeight="1">
-      <c r="A12" s="1" t="n"/>
-      <c r="B12" s="49" t="n"/>
-      <c r="C12" s="34" t="n"/>
-      <c r="D12" s="34" t="n"/>
-      <c r="E12" s="34" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G11" s="4"/>
+    </row>
+    <row r="12" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="1"/>
+      <c r="B12" s="49"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="34"/>
       <c r="F12" s="35">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
-        <v/>
-      </c>
-      <c r="G12" s="4" t="n"/>
-    </row>
-    <row r="13" ht="14.2" customHeight="1">
-      <c r="A13" s="1" t="n"/>
-      <c r="B13" s="49" t="n"/>
-      <c r="C13" s="34" t="n"/>
-      <c r="D13" s="34" t="n"/>
-      <c r="E13" s="34" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G12" s="4"/>
+    </row>
+    <row r="13" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="1"/>
+      <c r="B13" s="49"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="34"/>
       <c r="F13" s="35">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
-        <v/>
-      </c>
-      <c r="G13" s="4" t="n"/>
-    </row>
-    <row r="14" ht="14.2" customHeight="1">
-      <c r="A14" s="1" t="n"/>
-      <c r="B14" s="49" t="n"/>
-      <c r="C14" s="34" t="n"/>
-      <c r="D14" s="34" t="n"/>
-      <c r="E14" s="34" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="1"/>
+      <c r="B14" s="49"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="34"/>
+      <c r="E14" s="34"/>
       <c r="F14" s="35">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
-        <v/>
-      </c>
-      <c r="G14" s="4" t="n"/>
-    </row>
-    <row r="15" ht="14.2" customHeight="1">
-      <c r="A15" s="1" t="n"/>
-      <c r="B15" s="49" t="n"/>
-      <c r="C15" s="34" t="n"/>
-      <c r="D15" s="34" t="n"/>
-      <c r="E15" s="34" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G14" s="4"/>
+    </row>
+    <row r="15" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="1"/>
+      <c r="B15" s="49"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
       <c r="F15" s="35">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
-        <v/>
-      </c>
-      <c r="G15" s="4" t="n"/>
-    </row>
-    <row r="16" ht="14.2" customFormat="1" customHeight="1" s="12">
-      <c r="A16" s="1" t="n"/>
-      <c r="B16" s="49" t="n"/>
-      <c r="C16" s="34" t="n"/>
-      <c r="D16" s="34" t="n"/>
-      <c r="E16" s="34" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="1:7" s="12" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="1"/>
+      <c r="B16" s="49"/>
+      <c r="C16" s="34"/>
+      <c r="D16" s="34"/>
+      <c r="E16" s="34"/>
       <c r="F16" s="35">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
-        <v/>
-      </c>
-      <c r="G16" s="4" t="n"/>
-    </row>
-    <row r="17" ht="14.2" customFormat="1" customHeight="1" s="13">
-      <c r="A17" s="1" t="n"/>
-      <c r="B17" s="49" t="n"/>
-      <c r="C17" s="34" t="n"/>
-      <c r="D17" s="34" t="n"/>
-      <c r="E17" s="34" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="1"/>
+      <c r="B17" s="49"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="34"/>
       <c r="F17" s="35">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
-        <v/>
-      </c>
-      <c r="G17" s="4" t="n"/>
-    </row>
-    <row r="18" ht="14.2" customFormat="1" customHeight="1" s="13">
-      <c r="A18" s="2" t="n"/>
-      <c r="B18" s="49" t="n"/>
-      <c r="C18" s="34" t="n"/>
-      <c r="D18" s="34" t="n"/>
-      <c r="E18" s="34" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G17" s="4"/>
+    </row>
+    <row r="18" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="2"/>
+      <c r="B18" s="49"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
       <c r="F18" s="35">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
-        <v/>
-      </c>
-      <c r="G18" s="4" t="n"/>
-    </row>
-    <row r="19" ht="14.2" customFormat="1" customHeight="1" s="13">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="49" t="n"/>
-      <c r="C19" s="34" t="n"/>
-      <c r="D19" s="34" t="n"/>
-      <c r="E19" s="34" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G18" s="4"/>
+    </row>
+    <row r="19" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="2"/>
+      <c r="B19" s="49"/>
+      <c r="C19" s="34"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="34"/>
       <c r="F19" s="35">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
-        <v/>
-      </c>
-      <c r="G19" s="4" t="n"/>
-    </row>
-    <row r="20" ht="14.2" customFormat="1" customHeight="1" s="13">
-      <c r="A20" s="2" t="n"/>
-      <c r="B20" s="49" t="n"/>
-      <c r="C20" s="34" t="n"/>
-      <c r="D20" s="34" t="n"/>
-      <c r="E20" s="34" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G19" s="4"/>
+    </row>
+    <row r="20" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="2"/>
+      <c r="B20" s="49"/>
+      <c r="C20" s="34"/>
+      <c r="D20" s="34"/>
+      <c r="E20" s="34"/>
       <c r="F20" s="35">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
-        <v/>
-      </c>
-      <c r="G20" s="4" t="n"/>
-    </row>
-    <row r="21" ht="14.2" customFormat="1" customHeight="1" s="13">
-      <c r="A21" s="2" t="n"/>
-      <c r="B21" s="49" t="n"/>
-      <c r="C21" s="34" t="n"/>
-      <c r="D21" s="34" t="n"/>
-      <c r="E21" s="34" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G20" s="4"/>
+    </row>
+    <row r="21" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="2"/>
+      <c r="B21" s="49"/>
+      <c r="C21" s="34"/>
+      <c r="D21" s="34"/>
+      <c r="E21" s="34"/>
       <c r="F21" s="35">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
-        <v/>
-      </c>
-      <c r="G21" s="4" t="n"/>
-    </row>
-    <row r="22" ht="14.2" customFormat="1" customHeight="1" s="13">
-      <c r="A22" s="2" t="n"/>
-      <c r="B22" s="49" t="n"/>
-      <c r="C22" s="34" t="n"/>
-      <c r="D22" s="34" t="n"/>
-      <c r="E22" s="34" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G21" s="4"/>
+    </row>
+    <row r="22" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="2"/>
+      <c r="B22" s="49"/>
+      <c r="C22" s="34"/>
+      <c r="D22" s="34"/>
+      <c r="E22" s="34"/>
       <c r="F22" s="35">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
-        <v/>
-      </c>
-      <c r="G22" s="4" t="n"/>
-    </row>
-    <row r="23" ht="14.2" customFormat="1" customHeight="1" s="13">
-      <c r="A23" s="2" t="n"/>
-      <c r="B23" s="49" t="n"/>
-      <c r="C23" s="34" t="n"/>
-      <c r="D23" s="34" t="n"/>
-      <c r="E23" s="34" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G22" s="4"/>
+    </row>
+    <row r="23" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="2"/>
+      <c r="B23" s="49"/>
+      <c r="C23" s="34"/>
+      <c r="D23" s="34"/>
+      <c r="E23" s="34"/>
       <c r="F23" s="35">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
-        <v/>
-      </c>
-      <c r="G23" s="4" t="n"/>
-    </row>
-    <row r="24" ht="14.2" customFormat="1" customHeight="1" s="13">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="49" t="n"/>
-      <c r="C24" s="34" t="n"/>
-      <c r="D24" s="34" t="n"/>
-      <c r="E24" s="34" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G23" s="4"/>
+    </row>
+    <row r="24" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="2"/>
+      <c r="B24" s="49"/>
+      <c r="C24" s="34"/>
+      <c r="D24" s="34"/>
+      <c r="E24" s="34"/>
       <c r="F24" s="35">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
-        <v/>
-      </c>
-      <c r="G24" s="4" t="n"/>
-    </row>
-    <row r="25" ht="14.2" customFormat="1" customHeight="1" s="13">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="49" t="n"/>
-      <c r="C25" s="34" t="n"/>
-      <c r="D25" s="34" t="n"/>
-      <c r="E25" s="34" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G24" s="4"/>
+    </row>
+    <row r="25" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="2"/>
+      <c r="B25" s="49"/>
+      <c r="C25" s="34"/>
+      <c r="D25" s="34"/>
+      <c r="E25" s="34"/>
       <c r="F25" s="35">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
-        <v/>
-      </c>
-      <c r="G25" s="4" t="n"/>
-    </row>
-    <row r="26" ht="14.2" customFormat="1" customHeight="1" s="13">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="49" t="n"/>
-      <c r="C26" s="34" t="n"/>
-      <c r="D26" s="34" t="n"/>
-      <c r="E26" s="34" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G25" s="4"/>
+    </row>
+    <row r="26" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="2"/>
+      <c r="B26" s="49"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="34"/>
       <c r="F26" s="35">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
-        <v/>
-      </c>
-      <c r="G26" s="4" t="n"/>
-    </row>
-    <row r="27" ht="14.2" customFormat="1" customHeight="1" s="13">
-      <c r="A27" s="2" t="n"/>
-      <c r="B27" s="49" t="n"/>
-      <c r="C27" s="34" t="n"/>
-      <c r="D27" s="34" t="n"/>
-      <c r="E27" s="34" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G26" s="4"/>
+    </row>
+    <row r="27" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="2"/>
+      <c r="B27" s="49"/>
+      <c r="C27" s="34"/>
+      <c r="D27" s="34"/>
+      <c r="E27" s="34"/>
       <c r="F27" s="35">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
-        <v/>
-      </c>
-      <c r="G27" s="4" t="n"/>
-    </row>
-    <row r="28" ht="14.2" customFormat="1" customHeight="1" s="13">
-      <c r="A28" s="3" t="n"/>
-      <c r="B28" s="50" t="n"/>
-      <c r="C28" s="36" t="n"/>
-      <c r="D28" s="36" t="n"/>
-      <c r="E28" s="36" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G27" s="4"/>
+    </row>
+    <row r="28" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="3"/>
+      <c r="B28" s="50"/>
+      <c r="C28" s="36"/>
+      <c r="D28" s="36"/>
+      <c r="E28" s="36"/>
       <c r="F28" s="37">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
-        <v/>
-      </c>
-      <c r="G28" s="5" t="n"/>
-    </row>
-    <row r="29" ht="15.55" customFormat="1" customHeight="1" s="13">
-      <c r="A29" s="32" t="n"/>
-      <c r="B29" s="47" t="inlineStr">
-        <is>
-          <t>Insgesamt</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="G28" s="5"/>
+    </row>
+    <row r="29" spans="1:7" s="13" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="32"/>
+      <c r="B29" s="47" t="s">
+        <v>16</v>
       </c>
       <c r="C29" s="38">
         <f>ROUNDUP(SUBTOTAL(109,Tabelle1[Fahrtzeit])/5,0)*5</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D29" s="38">
         <f>ROUNDUP(SUBTOTAL(109,Tabelle1[Direkter Fallkontakt])/5,0)*5</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E29" s="38">
         <f>ROUNDUP(SUBTOTAL(109,Tabelle1[Indirekte Fallbearbeitung])/5,0)*5</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F29" s="39">
         <f>SUBTOTAL(109,Tabelle1[Summe Zeit])</f>
-        <v/>
-      </c>
-      <c r="G29" s="33" t="n"/>
-    </row>
-    <row r="30" ht="15.55" customFormat="1" customHeight="1" s="13">
-      <c r="A30" s="41" t="n"/>
-      <c r="B30" s="48" t="inlineStr">
-        <is>
-          <t>Obergrenze</t>
-        </is>
-      </c>
-      <c r="C30" s="44" t="n"/>
-      <c r="D30" s="44" t="n"/>
-      <c r="E30" s="44" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G29" s="33"/>
+    </row>
+    <row r="30" spans="1:7" s="13" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="41"/>
+      <c r="B30" s="48" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30" s="44"/>
+      <c r="D30" s="44"/>
+      <c r="E30" s="44"/>
       <c r="F30" s="45">
         <f>C30+D30+E30</f>
-        <v/>
-      </c>
-      <c r="G30" s="10" t="n"/>
-    </row>
-    <row r="31" ht="15.55" customFormat="1" customHeight="1" s="13">
-      <c r="A31" s="42" t="n"/>
-      <c r="B31" s="48" t="inlineStr">
-        <is>
-          <t>Differenz</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="G30" s="10"/>
+    </row>
+    <row r="31" spans="1:7" s="13" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="42"/>
+      <c r="B31" s="48" t="s">
+        <v>18</v>
       </c>
       <c r="C31" s="44">
         <f>C30-C29</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D31" s="46">
         <f>D30-D29</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E31" s="46">
         <f>E30-E29</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F31" s="46">
         <f>F30-F29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="31.3" customFormat="1" customHeight="1" s="13">
-      <c r="A32" s="43" t="n"/>
-      <c r="C32" s="43" t="n"/>
-      <c r="F32" s="43" t="n"/>
-    </row>
-    <row r="33" ht="15.55" customFormat="1" customHeight="1" s="13">
-      <c r="A33" s="11" t="n"/>
-      <c r="B33" s="11" t="n"/>
-      <c r="C33" s="11" t="n"/>
-      <c r="D33" s="11" t="n"/>
-      <c r="E33" s="11" t="n"/>
-      <c r="F33" s="11" t="n"/>
-      <c r="G33" s="11" t="n"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" s="13" customFormat="1" ht="31.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="43"/>
+      <c r="C32" s="43"/>
+      <c r="F32" s="43"/>
+    </row>
+    <row r="33" spans="1:7" s="13" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="11"/>
+      <c r="B33" s="11"/>
+      <c r="C33" s="11"/>
+      <c r="D33" s="11"/>
+      <c r="E33" s="11"/>
+      <c r="F33" s="11"/>
+      <c r="G33" s="11"/>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="NBfkXt6I5lXu3VlrBef8U4DD0nr6drmvpLDfuV8B8IhHEr5/XyofsWzaJqtZgWFv94sRtcelWgqMctYRHRYsJA==" saltValue="8LfnXzct7do3Vxdm8NGWJA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="4">
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A6:B6"/>
@@ -1930,29 +1948,37 @@
     <mergeCell ref="A5:B5"/>
   </mergeCells>
   <conditionalFormatting sqref="C31:F31">
-    <cfRule type="expression" priority="1" dxfId="21">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>C31&lt;0</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="22">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>AND(C31&gt;=0,C31&lt;0.2*C30)</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="23">
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>C31&gt;=0.2*C30</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="9"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
   <headerFooter differentFirst="1">
-    <oddHeader/>
-    <oddFooter>&amp;L&amp;9 Wegpiraten GmbH_x000a_Alpenstrasse 2_x000a_3800 Interlaken&amp;C&amp;9 Tel: 076 790 67 56_x000a_             E-Mail: info@wegpiraten.ch_x000a_ www.wegpiraten.ch&amp;R&amp;9 &amp;K000000Sozialpädagogische_x000a_Familienbegleitung&amp;K00+000A</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader>&amp;LV5.2 autom_x000a_&amp;RC3 - Vertraulich</firstHeader>
-    <firstFooter>&amp;L&amp;7 Wegpiraten GmbH_x000a_Hauptstraße 47_x000a_3800 Unterlakjen&amp;C&amp;7 Tel: 076 790 67 56_x000a_             E-Mail: info@wegpiraten.ch_x000a_ www.wegpiraten.ch&amp;R&amp;7 &amp;K000000Sozialpädagogische        &amp;K00+000A_x000a_Familienbegleitung          F</firstFooter>
+    <oddFooter>&amp;L&amp;9 Wegpiraten GmbH
+Alpenstrasse 2
+3800 Interlaken&amp;C&amp;9 Tel: 076 790 67 56
+             E-Mail: info@wegpiraten.ch
+ www.wegpiraten.ch&amp;R&amp;9 &amp;K000000Sozialpädagogische
+Familienbegleitung&amp;K00+000A</oddFooter>
+    <firstHeader>&amp;LV5.2 autom
+&amp;RC3 - Vertraulich</firstHeader>
+    <firstFooter>&amp;L&amp;7 Wegpiraten GmbH
+Hauptstraße 47
+3800 Unterlakjen&amp;C&amp;7 Tel: 076 790 67 56
+             E-Mail: info@wegpiraten.ch
+ www.wegpiraten.ch&amp;R&amp;7 &amp;K000000Sozialpädagogische        &amp;K00+000A
+Familienbegleitung          F</firstFooter>
   </headerFooter>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <drawing r:id="rId2"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Feature: Validierungslogik im Zeiterfassungsbogen-Template
- C32: WENN-Formel zeigt Warntext je Priorität (kein Zeilenumbruch)
  - Prio 1: "Budget überzogen!" wenn C31/D31/E31 negativ
  - Prio 2: "Zeiten für indirekte Fallbearbeitung überprüfen!" wenn E29 > 0.5*D29
- E29: Conditional Formatting (hellrot) wenn indirekte Summe > 50% der direkten Summe

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/time_sheet_template.xlsx
+++ b/templates/time_sheet_template.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Debian\home\stephan\projects\wegpiraten\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAF65A4C-E47F-42DA-B25C-0D9DA0A328FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{550ED12A-CBE2-4955-86A7-F33F77C081C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="9r/TxM3zBcSjnJTI/hP9y4R5VkDU9X45pyxBQ1SRhdgGa0G4N9+kmOzqUscJS/8FfSdUOZhKQAU6CU1O1OaWPA==" workbookSaltValue="Ey8SgEponXL1upYzdwO0ww==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="6390" windowWidth="38640" windowHeight="21120" tabRatio="709" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6480" yWindow="2780" windowWidth="28800" windowHeight="15290" tabRatio="709" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arbeitszeiterfassung" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,7 @@
     <t>Datum</t>
   </si>
   <si>
-    <t>Fahrtzeit</t>
+    <t>Fahrzeit</t>
   </si>
   <si>
     <t>Direkter Fallkontakt</t>
@@ -85,7 +85,7 @@
     <t>Insgesamt</t>
   </si>
   <si>
-    <t>Obergrenze</t>
+    <t>Soll</t>
   </si>
   <si>
     <t>Differenz</t>
@@ -360,7 +360,7 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="11"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="11"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="20" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
@@ -511,6 +511,9 @@
     <xf numFmtId="1" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -527,7 +530,15 @@
     <cellStyle name="Eingabe" xfId="1" builtinId="20"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="22">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="5" tint="0.59996337778862885"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1137,9 +1148,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>4562739</xdr:colOff>
+      <xdr:colOff>4559564</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>49392</xdr:rowOff>
+      <xdr:rowOff>46217</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1179,24 +1190,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A10:G29" totalsRowCount="1" headerRowDxfId="20" dataDxfId="19" totalsRowDxfId="17" tableBorderDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A10:G29" totalsRowCount="1" headerRowDxfId="21" dataDxfId="20" totalsRowDxfId="18" tableBorderDxfId="19">
   <autoFilter ref="A10:G28" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Uhrzeit" dataDxfId="16" totalsRowDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Datum" totalsRowLabel="Insgesamt" dataDxfId="14" totalsRowDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Fahrtzeit" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="11">
-      <totalsRowFormula>ROUNDUP(SUBTOTAL(109,Tabelle1[Fahrtzeit])/5,0)*5</totalsRowFormula>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Uhrzeit" dataDxfId="17" totalsRowDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Datum" totalsRowLabel="Insgesamt" dataDxfId="15" totalsRowDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Fahrzeit" totalsRowFunction="custom" dataDxfId="13" totalsRowDxfId="12">
+      <totalsRowFormula>ROUNDUP(SUBTOTAL(109,Tabelle1[Fahrzeit])/5,0)*5</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Direkter Fallkontakt" totalsRowFunction="custom" dataDxfId="10" totalsRowDxfId="9">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Direkter Fallkontakt" totalsRowFunction="custom" dataDxfId="11" totalsRowDxfId="10">
       <totalsRowFormula>ROUNDUP(SUBTOTAL(109,Tabelle1[Direkter Fallkontakt])/5,0)*5</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Indirekte Fallbearbeitung" totalsRowFunction="custom" dataDxfId="8" totalsRowDxfId="7">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Indirekte Fallbearbeitung" totalsRowFunction="custom" dataDxfId="9" totalsRowDxfId="8">
       <totalsRowFormula>ROUNDUP(SUBTOTAL(109,Tabelle1[Indirekte Fallbearbeitung])/5,0)*5</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Summe Zeit" totalsRowFunction="sum" dataDxfId="6" totalsRowDxfId="5">
-      <calculatedColumnFormula>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</calculatedColumnFormula>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Summe Zeit" totalsRowFunction="sum" dataDxfId="7" totalsRowDxfId="6">
+      <calculatedColumnFormula>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Notizen           " dataDxfId="4" totalsRowDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Notizen           " dataDxfId="5" totalsRowDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1559,10 +1570,11 @@
     <col min="2" max="2" width="11.26953125" style="7" customWidth="1"/>
     <col min="3" max="3" width="9.26953125" style="8" customWidth="1"/>
     <col min="4" max="4" width="12.90625" style="8" customWidth="1"/>
-    <col min="5" max="5" width="13.81640625" style="9" customWidth="1"/>
+    <col min="5" max="5" width="15.1796875" style="9" customWidth="1"/>
     <col min="6" max="6" width="12.81640625" style="8" customWidth="1"/>
     <col min="7" max="7" width="66.7265625" style="10" customWidth="1"/>
-    <col min="8" max="16384" width="11.26953125" style="11"/>
+    <col min="8" max="8" width="11.26953125" style="11" customWidth="1"/>
+    <col min="9" max="16384" width="11.26953125" style="11"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.5">
@@ -1574,10 +1586,10 @@
       </c>
     </row>
     <row r="5" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="54" t="s">
+      <c r="A5" s="55" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="55"/>
+      <c r="B5" s="56"/>
       <c r="C5" s="17"/>
       <c r="D5" s="17"/>
       <c r="E5" s="18" t="s">
@@ -1586,20 +1598,20 @@
       <c r="F5" s="19"/>
     </row>
     <row r="6" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="53" t="s">
+      <c r="A6" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="52"/>
+      <c r="B6" s="53"/>
       <c r="C6" s="20"/>
       <c r="D6" s="21"/>
       <c r="E6" s="18"/>
       <c r="F6" s="22"/>
     </row>
     <row r="7" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="53" t="s">
+      <c r="A7" s="54" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="52"/>
+      <c r="B7" s="53"/>
       <c r="C7" s="40"/>
       <c r="D7" s="23"/>
       <c r="E7" s="19" t="s">
@@ -1608,10 +1620,10 @@
       <c r="F7" s="22"/>
     </row>
     <row r="8" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="51" t="s">
+      <c r="A8" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="52"/>
+      <c r="B8" s="53"/>
       <c r="C8" s="21"/>
       <c r="D8" s="21"/>
       <c r="E8" s="22" t="s">
@@ -1627,7 +1639,7 @@
       <c r="E9" s="27"/>
       <c r="F9" s="26"/>
     </row>
-    <row r="10" spans="1:7" ht="24.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="29" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="28" t="s">
         <v>9</v>
       </c>
@@ -1657,7 +1669,7 @@
       <c r="D11" s="34"/>
       <c r="E11" s="34"/>
       <c r="F11" s="35">
-        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
       <c r="G11" s="4"/>
@@ -1669,7 +1681,7 @@
       <c r="D12" s="34"/>
       <c r="E12" s="34"/>
       <c r="F12" s="35">
-        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
       <c r="G12" s="4"/>
@@ -1681,7 +1693,7 @@
       <c r="D13" s="34"/>
       <c r="E13" s="34"/>
       <c r="F13" s="35">
-        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
       <c r="G13" s="4"/>
@@ -1693,7 +1705,7 @@
       <c r="D14" s="34"/>
       <c r="E14" s="34"/>
       <c r="F14" s="35">
-        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
       <c r="G14" s="4"/>
@@ -1705,7 +1717,7 @@
       <c r="D15" s="34"/>
       <c r="E15" s="34"/>
       <c r="F15" s="35">
-        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
       <c r="G15" s="4"/>
@@ -1717,7 +1729,7 @@
       <c r="D16" s="34"/>
       <c r="E16" s="34"/>
       <c r="F16" s="35">
-        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
       <c r="G16" s="4"/>
@@ -1729,7 +1741,7 @@
       <c r="D17" s="34"/>
       <c r="E17" s="34"/>
       <c r="F17" s="35">
-        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
       <c r="G17" s="4"/>
@@ -1741,7 +1753,7 @@
       <c r="D18" s="34"/>
       <c r="E18" s="34"/>
       <c r="F18" s="35">
-        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
       <c r="G18" s="4"/>
@@ -1753,7 +1765,7 @@
       <c r="D19" s="34"/>
       <c r="E19" s="34"/>
       <c r="F19" s="35">
-        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
       <c r="G19" s="4"/>
@@ -1765,7 +1777,7 @@
       <c r="D20" s="34"/>
       <c r="E20" s="34"/>
       <c r="F20" s="35">
-        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
       <c r="G20" s="4"/>
@@ -1777,7 +1789,7 @@
       <c r="D21" s="34"/>
       <c r="E21" s="34"/>
       <c r="F21" s="35">
-        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
       <c r="G21" s="4"/>
@@ -1789,7 +1801,7 @@
       <c r="D22" s="34"/>
       <c r="E22" s="34"/>
       <c r="F22" s="35">
-        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
       <c r="G22" s="4"/>
@@ -1801,7 +1813,7 @@
       <c r="D23" s="34"/>
       <c r="E23" s="34"/>
       <c r="F23" s="35">
-        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
       <c r="G23" s="4"/>
@@ -1813,7 +1825,7 @@
       <c r="D24" s="34"/>
       <c r="E24" s="34"/>
       <c r="F24" s="35">
-        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
       <c r="G24" s="4"/>
@@ -1825,7 +1837,7 @@
       <c r="D25" s="34"/>
       <c r="E25" s="34"/>
       <c r="F25" s="35">
-        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
       <c r="G25" s="4"/>
@@ -1837,7 +1849,7 @@
       <c r="D26" s="34"/>
       <c r="E26" s="34"/>
       <c r="F26" s="35">
-        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
       <c r="G26" s="4"/>
@@ -1849,7 +1861,7 @@
       <c r="D27" s="34"/>
       <c r="E27" s="34"/>
       <c r="F27" s="35">
-        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
       <c r="G27" s="4"/>
@@ -1861,7 +1873,7 @@
       <c r="D28" s="36"/>
       <c r="E28" s="36"/>
       <c r="F28" s="37">
-        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrtzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
+        <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
       <c r="G28" s="5"/>
@@ -1872,7 +1884,7 @@
         <v>16</v>
       </c>
       <c r="C29" s="38">
-        <f>ROUNDUP(SUBTOTAL(109,Tabelle1[Fahrtzeit])/5,0)*5</f>
+        <f>ROUNDUP(SUBTOTAL(109,Tabelle1[Fahrzeit])/5,0)*5</f>
         <v>0</v>
       </c>
       <c r="D29" s="38">
@@ -1925,9 +1937,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" s="13" customFormat="1" ht="31.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" s="13" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="43"/>
-      <c r="C32" s="43"/>
+      <c r="C32" s="51" t="str">
+        <f>IF(OR(C31&lt;0,D31&lt;0,E31&lt;0),"Budget überzogen! Prüfen und genehmigen lassen.",IF(E29&gt;0.5*D29,"Zeiten für indirekte Fallbearbeitung überprüfen!",""))</f>
+        <v/>
+      </c>
       <c r="F32" s="43"/>
     </row>
     <row r="33" spans="1:7" s="13" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1940,7 +1955,7 @@
       <c r="G33" s="11"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="NBfkXt6I5lXu3VlrBef8U4DD0nr6drmvpLDfuV8B8IhHEr5/XyofsWzaJqtZgWFv94sRtcelWgqMctYRHRYsJA==" saltValue="8LfnXzct7do3Vxdm8NGWJA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="bcW0jE250XslnwQSp2uAtheX7qQzgtad4YzUinzgMi+xnUP+0UuIx89/5R3QkbM/7qzy4iPtbkNi+HT86xFlXA==" saltValue="c0CBCfq1zxuvPmLD7j+H7w==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="4">
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A6:B6"/>
@@ -1948,14 +1963,19 @@
     <mergeCell ref="A5:B5"/>
   </mergeCells>
   <conditionalFormatting sqref="C31:F31">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>C31&lt;0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>AND(C31&gt;=0,C31&lt;0.2*C30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="1" priority="3">
       <formula>C31&gt;=0.2*C30</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E29">
+    <cfRule type="expression" dxfId="0" priority="7">
+      <formula>E29&gt;0.5*D29</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
@@ -1971,7 +1991,7 @@
 &amp;RC3 - Vertraulich</firstHeader>
     <firstFooter>&amp;L&amp;7 Wegpiraten GmbH
 Hauptstraße 47
-3800 Unterlakjen&amp;C&amp;7 Tel: 076 790 67 56
+3800 Unterseen&amp;C&amp;7 Tel: 076 790 67 56
              E-Mail: info@wegpiraten.ch
  www.wegpiraten.ch&amp;R&amp;7 &amp;K000000Sozialpädagogische        &amp;K00+000A
 Familienbegleitung          F</firstFooter>

</xml_diff>

<commit_message>
meldungen zur budgetüberziehung verschärft
</commit_message>
<xml_diff>
--- a/templates/time_sheet_template.xlsx
+++ b/templates/time_sheet_template.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Debian\home\stephan\projects\wegpiraten\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{550ED12A-CBE2-4955-86A7-F33F77C081C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2229543D-13F5-410E-B84E-F8C8E2738EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="9r/TxM3zBcSjnJTI/hP9y4R5VkDU9X45pyxBQ1SRhdgGa0G4N9+kmOzqUscJS/8FfSdUOZhKQAU6CU1O1OaWPA==" workbookSaltValue="Ey8SgEponXL1upYzdwO0ww==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="6480" yWindow="2780" windowWidth="28800" windowHeight="15290" tabRatio="709" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" tabRatio="709" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arbeitszeiterfassung" sheetId="1" r:id="rId1"/>
@@ -33,9 +33,6 @@
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
-  <si>
-    <t xml:space="preserve">        </t>
-  </si>
   <si>
     <t>Zeiterfassung</t>
   </si>
@@ -76,9 +73,6 @@
     <t>Indirekte Fallbearbeitung</t>
   </si>
   <si>
-    <t>Summe Zeit</t>
-  </si>
-  <si>
     <t xml:space="preserve">Notizen           </t>
   </si>
   <si>
@@ -90,18 +84,25 @@
   <si>
     <t>Differenz</t>
   </si>
+  <si>
+    <t>Summe h</t>
+  </si>
+  <si>
+    <t>Summe min</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="_ &quot;Fr.&quot;\ * #,##0.00_ ;_ &quot;Fr.&quot;\ * \-#,##0.00_ ;_ &quot;Fr.&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="165" formatCode="[$-407]mmmm\ yy;@"/>
     <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
     <numFmt numFmtId="167" formatCode="[h]&quot;h&quot;mm&quot;m&quot;"/>
+    <numFmt numFmtId="169" formatCode="[h]:mm"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -196,8 +197,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -214,8 +223,14 @@
         <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor theme="4" tint="0.59999389629810485"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -354,13 +369,28 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="11"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="11"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="20" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
@@ -404,7 +434,6 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -504,16 +533,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -524,21 +553,35 @@
       <alignment horizontal="left" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="15" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Berechnung" xfId="2" builtinId="22"/>
     <cellStyle name="Eingabe" xfId="1" builtinId="20"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="22">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="5" tint="0.59996337778862885"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="25">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -556,27 +599,291 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFCCCC"/>
-          <bgColor rgb="FFFFCCCC"/>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="5" tint="0.59996337778862885"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
+        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="10"/>
         <color auto="1"/>
         <name val="Calibri"/>
         <family val="2"/>
+        <scheme val="none"/>
       </font>
-      <alignment horizontal="left" vertical="bottom"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="169" formatCode="[h]:mm"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="169" formatCode="[h]:mm"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -612,34 +919,6 @@
         </bottom>
       </border>
       <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
-      <alignment horizontal="center" vertical="center"/>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
     </dxf>
     <dxf>
       <font>
@@ -682,7 +961,6 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
         <strike val="0"/>
         <condense val="0"/>
         <extend val="0"/>
@@ -695,17 +973,28 @@
         <family val="2"/>
       </font>
       <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
+      <fill>
+        <patternFill>
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="center"/>
-      <border outline="0">
+      <border>
         <left style="thin">
           <color indexed="64"/>
         </left>
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top/>
-        <bottom/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
       </border>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <font>
@@ -746,97 +1035,6 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
-      <alignment horizontal="center" vertical="center"/>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
-      <fill>
-        <patternFill>
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
-      <alignment horizontal="center" vertical="center"/>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
         <strike val="0"/>
         <condense val="0"/>
         <extend val="0"/>
@@ -885,30 +1083,7 @@
         <name val="Calibri"/>
         <family val="2"/>
       </font>
-      <alignment horizontal="right" vertical="bottom"/>
-      <border outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
+      <numFmt numFmtId="30" formatCode="@"/>
       <fill>
         <patternFill>
           <fgColor indexed="64"/>
@@ -931,21 +1106,6 @@
         </bottom>
       </border>
       <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom"/>
     </dxf>
     <dxf>
       <font>
@@ -1141,13 +1301,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>2732842</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>6350</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>4559564</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>46217</xdr:rowOff>
@@ -1190,24 +1350,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A10:G29" totalsRowCount="1" headerRowDxfId="21" dataDxfId="20" totalsRowDxfId="18" tableBorderDxfId="19">
-  <autoFilter ref="A10:G28" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Uhrzeit" dataDxfId="17" totalsRowDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Datum" totalsRowLabel="Insgesamt" dataDxfId="15" totalsRowDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Fahrzeit" totalsRowFunction="custom" dataDxfId="13" totalsRowDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A10:H29" totalsRowCount="1" headerRowDxfId="24" dataDxfId="23" totalsRowDxfId="21" tableBorderDxfId="22">
+  <autoFilter ref="A10:H28" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Uhrzeit" dataDxfId="20" totalsRowDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Datum" totalsRowLabel="Insgesamt" dataDxfId="19" totalsRowDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Fahrzeit" totalsRowFunction="custom" dataDxfId="18" totalsRowDxfId="10">
       <totalsRowFormula>ROUNDUP(SUBTOTAL(109,Tabelle1[Fahrzeit])/5,0)*5</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Direkter Fallkontakt" totalsRowFunction="custom" dataDxfId="11" totalsRowDxfId="10">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Direkter Fallkontakt" totalsRowFunction="custom" dataDxfId="17" totalsRowDxfId="9">
       <totalsRowFormula>ROUNDUP(SUBTOTAL(109,Tabelle1[Direkter Fallkontakt])/5,0)*5</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Indirekte Fallbearbeitung" totalsRowFunction="custom" dataDxfId="9" totalsRowDxfId="8">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Indirekte Fallbearbeitung" totalsRowFunction="custom" dataDxfId="16" totalsRowDxfId="8">
       <totalsRowFormula>ROUNDUP(SUBTOTAL(109,Tabelle1[Indirekte Fallbearbeitung])/5,0)*5</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Summe Zeit" totalsRowFunction="sum" dataDxfId="7" totalsRowDxfId="6">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Summe min" totalsRowFunction="sum" dataDxfId="15" totalsRowDxfId="7">
       <calculatedColumnFormula>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Notizen           " dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{AC106A25-B6EE-49FC-BF75-19497D970AE3}" name="Summe h" totalsRowFunction="custom" dataDxfId="13" totalsRowDxfId="6">
+      <calculatedColumnFormula>Tabelle1[[#This Row],[Summe min]]/1440</calculatedColumnFormula>
+      <totalsRowFormula>Tabelle1[[#Totals],[Summe min]]/1440</totalsRowFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Notizen           " dataDxfId="14" totalsRowDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1563,419 +1727,521 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A3:G33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.26953125" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
+  <dimension ref="A3:H34"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.27734375" defaultRowHeight="12.9" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="11.81640625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="11.26953125" style="7" customWidth="1"/>
-    <col min="3" max="3" width="9.26953125" style="8" customWidth="1"/>
-    <col min="4" max="4" width="12.90625" style="8" customWidth="1"/>
-    <col min="5" max="5" width="15.1796875" style="9" customWidth="1"/>
-    <col min="6" max="6" width="12.81640625" style="8" customWidth="1"/>
-    <col min="7" max="7" width="66.7265625" style="10" customWidth="1"/>
-    <col min="8" max="8" width="11.26953125" style="11" customWidth="1"/>
-    <col min="9" max="16384" width="11.26953125" style="11"/>
+    <col min="1" max="1" width="11.83203125" style="6" customWidth="1"/>
+    <col min="2" max="2" width="11.27734375" style="7" customWidth="1"/>
+    <col min="3" max="3" width="9.27734375" style="8" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" style="8" customWidth="1"/>
+    <col min="5" max="5" width="15.1640625" style="9" customWidth="1"/>
+    <col min="6" max="6" width="9" style="8" customWidth="1"/>
+    <col min="7" max="7" width="7.5546875" style="8" customWidth="1"/>
+    <col min="8" max="8" width="66.71875" style="10" customWidth="1"/>
+    <col min="9" max="9" width="11.27734375" style="11" customWidth="1"/>
+    <col min="10" max="16384" width="11.27734375" style="11"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.8">
       <c r="A3" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="16" t="s">
+    </row>
+    <row r="5" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="54" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="55" t="s">
+      <c r="B5" s="55"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="56"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="18" t="s">
+      <c r="F5" s="18"/>
+      <c r="G5" s="56"/>
+    </row>
+    <row r="6" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A6" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="F5" s="19"/>
-    </row>
-    <row r="6" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="54" t="s">
+      <c r="B6" s="52"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="57"/>
+    </row>
+    <row r="7" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A7" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="53"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="22"/>
-    </row>
-    <row r="7" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="54" t="s">
+      <c r="B7" s="52"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="53"/>
-      <c r="C7" s="40"/>
-      <c r="D7" s="23"/>
-      <c r="E7" s="19" t="s">
+      <c r="F7" s="21"/>
+      <c r="G7" s="57"/>
+    </row>
+    <row r="8" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="F7" s="22"/>
-    </row>
-    <row r="8" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="52" t="s">
+      <c r="B8" s="52"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="53"/>
-      <c r="C8" s="21"/>
-      <c r="D8" s="21"/>
-      <c r="E8" s="22" t="s">
+      <c r="F8" s="21"/>
+      <c r="G8" s="57"/>
+    </row>
+    <row r="9" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="23"/>
+      <c r="B9" s="24"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="59"/>
+    </row>
+    <row r="10" spans="1:8" ht="29.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A10" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="22"/>
-    </row>
-    <row r="9" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="24"/>
-      <c r="B9" s="25"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="26"/>
-    </row>
-    <row r="10" spans="1:7" ht="29" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="28" t="s">
+      <c r="B10" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="C10" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="28" t="s">
+      <c r="D10" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="28" t="s">
+      <c r="E10" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="30" t="s">
+      <c r="F10" s="30" t="s">
+        <v>18</v>
+      </c>
+      <c r="G10" s="30" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="F10" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="G10" s="28" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A11" s="14"/>
       <c r="B11" s="49"/>
-      <c r="C11" s="34"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="35">
+      <c r="C11" s="33"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="33"/>
+      <c r="F11" s="34">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="4"/>
-    </row>
-    <row r="12" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G11" s="58">
+        <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="4"/>
+    </row>
+    <row r="12" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A12" s="1"/>
       <c r="B12" s="49"/>
-      <c r="C12" s="34"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="34"/>
-      <c r="F12" s="35">
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="33"/>
+      <c r="F12" s="34">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G12" s="4"/>
-    </row>
-    <row r="13" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G12" s="58">
+        <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="4"/>
+    </row>
+    <row r="13" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A13" s="1"/>
       <c r="B13" s="49"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="35">
+      <c r="C13" s="33"/>
+      <c r="D13" s="33"/>
+      <c r="E13" s="33"/>
+      <c r="F13" s="34">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G13" s="4"/>
-    </row>
-    <row r="14" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G13" s="58">
+        <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="4"/>
+    </row>
+    <row r="14" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A14" s="1"/>
       <c r="B14" s="49"/>
-      <c r="C14" s="34"/>
-      <c r="D14" s="34"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="35">
+      <c r="C14" s="33"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="33"/>
+      <c r="F14" s="34">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="4"/>
-    </row>
-    <row r="15" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G14" s="58">
+        <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H14" s="4"/>
+    </row>
+    <row r="15" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A15" s="1"/>
       <c r="B15" s="49"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="35">
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="33"/>
+      <c r="F15" s="34">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G15" s="4"/>
-    </row>
-    <row r="16" spans="1:7" s="12" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G15" s="58">
+        <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="4"/>
+    </row>
+    <row r="16" spans="1:8" s="12" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A16" s="1"/>
       <c r="B16" s="49"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="35">
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="34">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G16" s="4"/>
-    </row>
-    <row r="17" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G16" s="58">
+        <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="4"/>
+    </row>
+    <row r="17" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A17" s="1"/>
       <c r="B17" s="49"/>
-      <c r="C17" s="34"/>
-      <c r="D17" s="34"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="35">
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="34">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G17" s="4"/>
-    </row>
-    <row r="18" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G17" s="58">
+        <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H17" s="4"/>
+    </row>
+    <row r="18" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A18" s="2"/>
       <c r="B18" s="49"/>
-      <c r="C18" s="34"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="35">
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="34">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G18" s="4"/>
-    </row>
-    <row r="19" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G18" s="58">
+        <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H18" s="4"/>
+    </row>
+    <row r="19" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A19" s="2"/>
       <c r="B19" s="49"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="35">
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="34">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G19" s="4"/>
-    </row>
-    <row r="20" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G19" s="58">
+        <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H19" s="4"/>
+    </row>
+    <row r="20" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A20" s="2"/>
       <c r="B20" s="49"/>
-      <c r="C20" s="34"/>
-      <c r="D20" s="34"/>
-      <c r="E20" s="34"/>
-      <c r="F20" s="35">
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="34">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G20" s="4"/>
-    </row>
-    <row r="21" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G20" s="58">
+        <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H20" s="4"/>
+    </row>
+    <row r="21" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A21" s="2"/>
       <c r="B21" s="49"/>
-      <c r="C21" s="34"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="34"/>
-      <c r="F21" s="35">
+      <c r="C21" s="33"/>
+      <c r="D21" s="33"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="34">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G21" s="4"/>
-    </row>
-    <row r="22" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G21" s="58">
+        <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H21" s="4"/>
+    </row>
+    <row r="22" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A22" s="2"/>
       <c r="B22" s="49"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="34"/>
-      <c r="E22" s="34"/>
-      <c r="F22" s="35">
+      <c r="C22" s="33"/>
+      <c r="D22" s="62"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="34">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G22" s="4"/>
-    </row>
-    <row r="23" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G22" s="58">
+        <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H22" s="4"/>
+    </row>
+    <row r="23" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A23" s="2"/>
       <c r="B23" s="49"/>
-      <c r="C23" s="34"/>
-      <c r="D23" s="34"/>
-      <c r="E23" s="34"/>
-      <c r="F23" s="35">
+      <c r="C23" s="33"/>
+      <c r="D23" s="33"/>
+      <c r="E23" s="33"/>
+      <c r="F23" s="34">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G23" s="4"/>
-    </row>
-    <row r="24" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G23" s="58">
+        <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H23" s="4"/>
+    </row>
+    <row r="24" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A24" s="2"/>
       <c r="B24" s="49"/>
-      <c r="C24" s="34"/>
-      <c r="D24" s="34"/>
-      <c r="E24" s="34"/>
-      <c r="F24" s="35">
+      <c r="C24" s="33"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="34">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G24" s="4"/>
-    </row>
-    <row r="25" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G24" s="58">
+        <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="4"/>
+    </row>
+    <row r="25" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A25" s="2"/>
       <c r="B25" s="49"/>
-      <c r="C25" s="34"/>
-      <c r="D25" s="34"/>
-      <c r="E25" s="34"/>
-      <c r="F25" s="35">
+      <c r="C25" s="33"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="34">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G25" s="4"/>
-    </row>
-    <row r="26" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G25" s="58">
+        <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="4"/>
+    </row>
+    <row r="26" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A26" s="2"/>
       <c r="B26" s="49"/>
-      <c r="C26" s="34"/>
-      <c r="D26" s="34"/>
-      <c r="E26" s="34"/>
-      <c r="F26" s="35">
+      <c r="C26" s="33"/>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="34">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G26" s="4"/>
-    </row>
-    <row r="27" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G26" s="58">
+        <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="4"/>
+    </row>
+    <row r="27" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A27" s="2"/>
       <c r="B27" s="49"/>
-      <c r="C27" s="34"/>
-      <c r="D27" s="34"/>
-      <c r="E27" s="34"/>
-      <c r="F27" s="35">
+      <c r="C27" s="33"/>
+      <c r="D27" s="33"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="34">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G27" s="4"/>
-    </row>
-    <row r="28" spans="1:7" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G27" s="58">
+        <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="4"/>
+    </row>
+    <row r="28" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A28" s="3"/>
       <c r="B28" s="50"/>
-      <c r="C28" s="36"/>
-      <c r="D28" s="36"/>
-      <c r="E28" s="36"/>
-      <c r="F28" s="37">
+      <c r="C28" s="35"/>
+      <c r="D28" s="35"/>
+      <c r="E28" s="35"/>
+      <c r="F28" s="36">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G28" s="5"/>
-    </row>
-    <row r="29" spans="1:7" s="13" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="32"/>
-      <c r="B29" s="47" t="s">
+      <c r="G28" s="60">
+        <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H28" s="5"/>
+    </row>
+    <row r="29" spans="1:8" s="13" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A29" s="31"/>
+      <c r="B29" s="46" t="s">
+        <v>14</v>
+      </c>
+      <c r="C29" s="37">
+        <f>ROUNDUP(SUBTOTAL(109,Tabelle1[Fahrzeit])/5,0)*5</f>
+        <v>0</v>
+      </c>
+      <c r="D29" s="37">
+        <f>ROUNDUP(SUBTOTAL(109,Tabelle1[Direkter Fallkontakt])/5,0)*5</f>
+        <v>0</v>
+      </c>
+      <c r="E29" s="37">
+        <f>ROUNDUP(SUBTOTAL(109,Tabelle1[Indirekte Fallbearbeitung])/5,0)*5</f>
+        <v>0</v>
+      </c>
+      <c r="F29" s="38">
+        <f>SUBTOTAL(109,Tabelle1[Summe min])</f>
+        <v>0</v>
+      </c>
+      <c r="G29" s="61">
+        <f>Tabelle1[[#Totals],[Summe min]]/1440</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="32"/>
+    </row>
+    <row r="30" spans="1:8" s="13" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A30" s="40"/>
+      <c r="B30" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="44">
+        <f>C30+D30+E30</f>
+        <v>0</v>
+      </c>
+      <c r="G30" s="44"/>
+      <c r="H30" s="10"/>
+    </row>
+    <row r="31" spans="1:8" s="13" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A31" s="41"/>
+      <c r="B31" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="C29" s="38">
-        <f>ROUNDUP(SUBTOTAL(109,Tabelle1[Fahrzeit])/5,0)*5</f>
-        <v>0</v>
-      </c>
-      <c r="D29" s="38">
-        <f>ROUNDUP(SUBTOTAL(109,Tabelle1[Direkter Fallkontakt])/5,0)*5</f>
-        <v>0</v>
-      </c>
-      <c r="E29" s="38">
-        <f>ROUNDUP(SUBTOTAL(109,Tabelle1[Indirekte Fallbearbeitung])/5,0)*5</f>
-        <v>0</v>
-      </c>
-      <c r="F29" s="39">
-        <f>SUBTOTAL(109,Tabelle1[Summe Zeit])</f>
-        <v>0</v>
-      </c>
-      <c r="G29" s="33"/>
-    </row>
-    <row r="30" spans="1:7" s="13" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="41"/>
-      <c r="B30" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="C30" s="44"/>
-      <c r="D30" s="44"/>
-      <c r="E30" s="44"/>
-      <c r="F30" s="45">
-        <f>C30+D30+E30</f>
-        <v>0</v>
-      </c>
-      <c r="G30" s="10"/>
-    </row>
-    <row r="31" spans="1:7" s="13" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="42"/>
-      <c r="B31" s="48" t="s">
-        <v>18</v>
-      </c>
-      <c r="C31" s="44">
+      <c r="C31" s="43">
         <f>C30-C29</f>
         <v>0</v>
       </c>
-      <c r="D31" s="46">
+      <c r="D31" s="45">
         <f>D30-D29</f>
         <v>0</v>
       </c>
-      <c r="E31" s="46">
+      <c r="E31" s="45">
         <f>E30-E29</f>
         <v>0</v>
       </c>
-      <c r="F31" s="46">
+      <c r="F31" s="45">
         <f>F30-F29</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" s="13" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="43"/>
-      <c r="C32" s="51" t="str">
+      <c r="G31" s="45"/>
+    </row>
+    <row r="32" spans="1:8" s="13" customFormat="1" ht="8.5" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A32" s="41"/>
+      <c r="B32" s="47"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="45"/>
+      <c r="E32" s="45"/>
+      <c r="F32" s="45"/>
+      <c r="G32" s="45"/>
+    </row>
+    <row r="33" spans="1:8" s="13" customFormat="1" ht="15.6" x14ac:dyDescent="0.6">
+      <c r="A33" s="42"/>
+      <c r="C33" s="48" t="str">
         <f>IF(OR(C31&lt;0,D31&lt;0,E31&lt;0),"Budget überzogen! Prüfen und genehmigen lassen.",IF(E29&gt;0.5*D29,"Zeiten für indirekte Fallbearbeitung überprüfen!",""))</f>
         <v/>
       </c>
-      <c r="F32" s="43"/>
-    </row>
-    <row r="33" spans="1:7" s="13" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="11"/>
-      <c r="B33" s="11"/>
-      <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="11"/>
-      <c r="F33" s="11"/>
-      <c r="G33" s="11"/>
+      <c r="D33" s="48"/>
+      <c r="E33" s="48"/>
+      <c r="F33" s="48"/>
+      <c r="G33" s="48"/>
+    </row>
+    <row r="34" spans="1:8" s="13" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A34" s="11"/>
+      <c r="B34" s="11"/>
+      <c r="C34" s="11"/>
+      <c r="D34" s="11"/>
+      <c r="E34" s="11"/>
+      <c r="F34" s="11"/>
+      <c r="G34" s="11"/>
+      <c r="H34" s="11"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="bcW0jE250XslnwQSp2uAtheX7qQzgtad4YzUinzgMi+xnUP+0UuIx89/5R3QkbM/7qzy4iPtbkNi+HT86xFlXA==" saltValue="c0CBCfq1zxuvPmLD7j+H7w==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="3QcLdSrvkVhIVnK36IghcSCivjGKP9GdF5KQ3ujOk9FBSupo+ya0i2e7/FsHCSqZSJZJ0mMUUpJAiNcTDq6o+A==" saltValue="IxK/hi5LX/tu/tCGlX+vLg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="4">
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A5:B5"/>
   </mergeCells>
+  <conditionalFormatting sqref="E29">
+    <cfRule type="expression" dxfId="4" priority="9">
+      <formula>E29&gt;0.5*D29</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C33:G33">
+    <cfRule type="expression" dxfId="3" priority="2">
+      <formula>LEN($C$33)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C31:F31">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>C31&lt;0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="1" priority="4">
       <formula>AND(C31&gt;=0,C31&lt;0.2*C30)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="3">
+    <cfRule type="expression" dxfId="0" priority="5">
       <formula>C31&gt;=0.2*C30</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E29">
-    <cfRule type="expression" dxfId="0" priority="7">
-      <formula>E29&gt;0.5*D29</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
@@ -1989,12 +2255,6 @@
 Familienbegleitung&amp;K00+000A</oddFooter>
     <firstHeader>&amp;LV5.2 autom
 &amp;RC3 - Vertraulich</firstHeader>
-    <firstFooter>&amp;L&amp;7 Wegpiraten GmbH
-Hauptstraße 47
-3800 Unterseen&amp;C&amp;7 Tel: 076 790 67 56
-             E-Mail: info@wegpiraten.ch
- www.wegpiraten.ch&amp;R&amp;7 &amp;K000000Sozialpädagogische        &amp;K00+000A
-Familienbegleitung          F</firstFooter>
   </headerFooter>
   <drawing r:id="rId2"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Fix Vorschau-Summe und aktualisiere Timesheet-Template
</commit_message>
<xml_diff>
--- a/templates/time_sheet_template.xlsx
+++ b/templates/time_sheet_template.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Debian\home\stephan\projects\wegpiraten\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2229543D-13F5-410E-B84E-F8C8E2738EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3EBCC4B-8D39-4D1B-BF4B-B9E9E5E7B078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="9r/TxM3zBcSjnJTI/hP9y4R5VkDU9X45pyxBQ1SRhdgGa0G4N9+kmOzqUscJS/8FfSdUOZhKQAU6CU1O1OaWPA==" workbookSaltValue="Ey8SgEponXL1upYzdwO0ww==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" tabRatio="709" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="6390" windowWidth="38640" windowHeight="21120" tabRatio="709" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arbeitszeiterfassung" sheetId="1" r:id="rId1"/>
@@ -100,9 +100,9 @@
     <numFmt numFmtId="165" formatCode="[$-407]mmmm\ yy;@"/>
     <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
     <numFmt numFmtId="167" formatCode="[h]&quot;h&quot;mm&quot;m&quot;"/>
-    <numFmt numFmtId="169" formatCode="[h]:mm"/>
+    <numFmt numFmtId="168" formatCode="[h]:mm"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -197,16 +197,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -223,14 +215,8 @@
         <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor theme="4" tint="0.59999389629810485"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -369,28 +355,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color theme="0"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="11"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="11"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="20" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
@@ -544,6 +515,25 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -553,28 +543,6 @@
       <alignment horizontal="left" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="15" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Berechnung" xfId="2" builtinId="22"/>
@@ -583,22 +551,6 @@
   </cellStyles>
   <dxfs count="25">
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB3FFD9"/>
-          <bgColor rgb="FFB3FFD9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF99"/>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -606,7 +558,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFFCCCC"/>
+          <fgColor theme="5" tint="0.59996337778862885"/>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -624,6 +576,22 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB3FFD9"/>
+          <bgColor rgb="FFB3FFD9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF99"/>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -631,7 +599,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="5" tint="0.59996337778862885"/>
+          <fgColor rgb="FFFFCCCC"/>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -654,236 +622,6 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="169" formatCode="[h]:mm"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="169" formatCode="[h]:mm"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
     </dxf>
     <dxf>
       <font>
@@ -919,6 +657,100 @@
         </bottom>
       </border>
       <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="168" formatCode="[h]:mm"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="168" formatCode="[h]:mm"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -961,40 +793,33 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
+        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="10"/>
         <color auto="1"/>
         <name val="Calibri"/>
         <family val="2"/>
+        <scheme val="none"/>
       </font>
       <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
-      <fill>
-        <patternFill>
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center"/>
-      <border>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <top/>
+        <bottom/>
       </border>
-      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1035,6 +860,103 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
+      <fill>
+        <patternFill>
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0&quot; min&quot;"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
         <strike val="0"/>
         <condense val="0"/>
         <extend val="0"/>
@@ -1069,6 +991,33 @@
         </bottom>
       </border>
       <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1106,6 +1055,25 @@
         </bottom>
       </border>
       <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1302,15 +1270,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>2732842</xdr:colOff>
+      <xdr:colOff>2556390</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>6350</xdr:rowOff>
+      <xdr:rowOff>6446</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>4559564</xdr:colOff>
+      <xdr:colOff>4383112</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>46217</xdr:rowOff>
+      <xdr:rowOff>49488</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1333,8 +1301,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7781092" y="6350"/>
-          <a:ext cx="1829897" cy="1528942"/>
+          <a:off x="7934648" y="6446"/>
+          <a:ext cx="1826722" cy="1540776"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1351,27 +1319,26 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A10:H29" totalsRowCount="1" headerRowDxfId="24" dataDxfId="23" totalsRowDxfId="21" tableBorderDxfId="22">
-  <autoFilter ref="A10:H28" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Uhrzeit" dataDxfId="20" totalsRowDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Datum" totalsRowLabel="Insgesamt" dataDxfId="19" totalsRowDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Fahrzeit" totalsRowFunction="custom" dataDxfId="18" totalsRowDxfId="10">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Uhrzeit" dataDxfId="20" totalsRowDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Datum" totalsRowLabel="Insgesamt" dataDxfId="18" totalsRowDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Fahrzeit" totalsRowFunction="custom" dataDxfId="16" totalsRowDxfId="15">
       <totalsRowFormula>ROUNDUP(SUBTOTAL(109,Tabelle1[Fahrzeit])/5,0)*5</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Direkter Fallkontakt" totalsRowFunction="custom" dataDxfId="17" totalsRowDxfId="9">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Direkter Fallkontakt" totalsRowFunction="custom" dataDxfId="14" totalsRowDxfId="13">
       <totalsRowFormula>ROUNDUP(SUBTOTAL(109,Tabelle1[Direkter Fallkontakt])/5,0)*5</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Indirekte Fallbearbeitung" totalsRowFunction="custom" dataDxfId="16" totalsRowDxfId="8">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Indirekte Fallbearbeitung" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="11">
       <totalsRowFormula>ROUNDUP(SUBTOTAL(109,Tabelle1[Indirekte Fallbearbeitung])/5,0)*5</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Summe min" totalsRowFunction="sum" dataDxfId="15" totalsRowDxfId="7">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Summe min" totalsRowFunction="sum" dataDxfId="10" totalsRowDxfId="9">
       <calculatedColumnFormula>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{AC106A25-B6EE-49FC-BF75-19497D970AE3}" name="Summe h" totalsRowFunction="custom" dataDxfId="13" totalsRowDxfId="6">
+    <tableColumn id="4" xr3:uid="{AC106A25-B6EE-49FC-BF75-19497D970AE3}" name="Summe h" totalsRowFunction="custom" dataDxfId="8" totalsRowDxfId="7">
       <calculatedColumnFormula>Tabelle1[[#This Row],[Summe min]]/1440</calculatedColumnFormula>
       <totalsRowFormula>Tabelle1[[#Totals],[Summe min]]/1440</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Notizen           " dataDxfId="14" totalsRowDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Notizen           " dataDxfId="6" totalsRowDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1728,85 +1695,84 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A3:H34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.27734375" defaultRowHeight="12.9" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.26953125" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.83203125" style="6" customWidth="1"/>
-    <col min="2" max="2" width="11.27734375" style="7" customWidth="1"/>
-    <col min="3" max="3" width="9.27734375" style="8" customWidth="1"/>
-    <col min="4" max="4" width="12.88671875" style="8" customWidth="1"/>
-    <col min="5" max="5" width="15.1640625" style="9" customWidth="1"/>
+    <col min="1" max="1" width="11.81640625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="11.26953125" style="7" customWidth="1"/>
+    <col min="3" max="3" width="9.26953125" style="8" customWidth="1"/>
+    <col min="4" max="4" width="12.90625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="15.1796875" style="9" customWidth="1"/>
     <col min="6" max="6" width="9" style="8" customWidth="1"/>
-    <col min="7" max="7" width="7.5546875" style="8" customWidth="1"/>
-    <col min="8" max="8" width="66.71875" style="10" customWidth="1"/>
-    <col min="9" max="9" width="11.27734375" style="11" customWidth="1"/>
-    <col min="10" max="16384" width="11.27734375" style="11"/>
+    <col min="7" max="7" width="7.54296875" style="8" customWidth="1"/>
+    <col min="8" max="8" width="64.08984375" style="10" customWidth="1"/>
+    <col min="9" max="16384" width="11.26953125" style="11"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.8">
+    <row r="3" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A3" s="15" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="54" t="s">
+    <row r="5" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="60" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="55"/>
+      <c r="B5" s="61"/>
       <c r="C5" s="16"/>
       <c r="D5" s="16"/>
       <c r="E5" s="17" t="s">
         <v>2</v>
       </c>
       <c r="F5" s="18"/>
-      <c r="G5" s="56"/>
-    </row>
-    <row r="6" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A6" s="53" t="s">
+      <c r="G5" s="51"/>
+    </row>
+    <row r="6" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="52"/>
+      <c r="B6" s="58"/>
       <c r="C6" s="19"/>
       <c r="D6" s="20"/>
       <c r="E6" s="17"/>
       <c r="F6" s="21"/>
-      <c r="G6" s="57"/>
-    </row>
-    <row r="7" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A7" s="53" t="s">
+      <c r="G6" s="52"/>
+    </row>
+    <row r="7" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="52"/>
+      <c r="B7" s="58"/>
       <c r="C7" s="39"/>
       <c r="D7" s="22"/>
       <c r="E7" s="18" t="s">
         <v>5</v>
       </c>
       <c r="F7" s="21"/>
-      <c r="G7" s="57"/>
-    </row>
-    <row r="8" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="51" t="s">
+      <c r="G7" s="52"/>
+    </row>
+    <row r="8" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="57" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="52"/>
+      <c r="B8" s="58"/>
       <c r="C8" s="20"/>
       <c r="D8" s="20"/>
       <c r="E8" s="21" t="s">
         <v>7</v>
       </c>
       <c r="F8" s="21"/>
-      <c r="G8" s="57"/>
-    </row>
-    <row r="9" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="G8" s="52"/>
+    </row>
+    <row r="9" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="23"/>
       <c r="B9" s="24"/>
       <c r="C9" s="25"/>
       <c r="D9" s="25"/>
       <c r="E9" s="26"/>
       <c r="F9" s="25"/>
-      <c r="G9" s="59"/>
-    </row>
-    <row r="10" spans="1:8" ht="29.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="G9" s="11"/>
+    </row>
+    <row r="10" spans="1:8" ht="29" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="27" t="s">
         <v>8</v>
       </c>
@@ -1832,7 +1798,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14"/>
       <c r="B11" s="49"/>
       <c r="C11" s="33"/>
@@ -1842,13 +1808,13 @@
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="58">
+      <c r="G11" s="53">
         <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H11" s="4"/>
     </row>
-    <row r="12" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="49"/>
       <c r="C12" s="33"/>
@@ -1858,13 +1824,13 @@
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G12" s="58">
+      <c r="G12" s="53">
         <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H12" s="4"/>
     </row>
-    <row r="13" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="49"/>
       <c r="C13" s="33"/>
@@ -1874,13 +1840,13 @@
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G13" s="58">
+      <c r="G13" s="53">
         <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H13" s="4"/>
     </row>
-    <row r="14" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="49"/>
       <c r="C14" s="33"/>
@@ -1890,13 +1856,13 @@
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="58">
+      <c r="G14" s="53">
         <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H14" s="4"/>
     </row>
-    <row r="15" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="49"/>
       <c r="C15" s="33"/>
@@ -1906,13 +1872,13 @@
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G15" s="58">
+      <c r="G15" s="53">
         <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H15" s="4"/>
     </row>
-    <row r="16" spans="1:8" s="12" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="16" spans="1:8" s="12" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
       <c r="B16" s="49"/>
       <c r="C16" s="33"/>
@@ -1922,13 +1888,13 @@
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G16" s="58">
+      <c r="G16" s="53">
         <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H16" s="4"/>
     </row>
-    <row r="17" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="17" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
       <c r="B17" s="49"/>
       <c r="C17" s="33"/>
@@ -1938,13 +1904,13 @@
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G17" s="58">
+      <c r="G17" s="53">
         <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H17" s="4"/>
     </row>
-    <row r="18" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="18" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2"/>
       <c r="B18" s="49"/>
       <c r="C18" s="33"/>
@@ -1954,13 +1920,13 @@
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G18" s="58">
+      <c r="G18" s="53">
         <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H18" s="4"/>
     </row>
-    <row r="19" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="19" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2"/>
       <c r="B19" s="49"/>
       <c r="C19" s="33"/>
@@ -1970,13 +1936,13 @@
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G19" s="58">
+      <c r="G19" s="53">
         <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H19" s="4"/>
     </row>
-    <row r="20" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="20" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2"/>
       <c r="B20" s="49"/>
       <c r="C20" s="33"/>
@@ -1986,13 +1952,13 @@
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G20" s="58">
+      <c r="G20" s="53">
         <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H20" s="4"/>
     </row>
-    <row r="21" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="21" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="2"/>
       <c r="B21" s="49"/>
       <c r="C21" s="33"/>
@@ -2002,29 +1968,29 @@
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G21" s="58">
+      <c r="G21" s="53">
         <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H21" s="4"/>
     </row>
-    <row r="22" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="22" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2"/>
       <c r="B22" s="49"/>
       <c r="C22" s="33"/>
-      <c r="D22" s="62"/>
+      <c r="D22" s="56"/>
       <c r="E22" s="33"/>
       <c r="F22" s="34">
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G22" s="58">
+      <c r="G22" s="53">
         <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H22" s="4"/>
     </row>
-    <row r="23" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="23" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="2"/>
       <c r="B23" s="49"/>
       <c r="C23" s="33"/>
@@ -2034,13 +2000,13 @@
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G23" s="58">
+      <c r="G23" s="53">
         <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H23" s="4"/>
     </row>
-    <row r="24" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="24" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2"/>
       <c r="B24" s="49"/>
       <c r="C24" s="33"/>
@@ -2050,13 +2016,13 @@
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G24" s="58">
+      <c r="G24" s="53">
         <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H24" s="4"/>
     </row>
-    <row r="25" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="25" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2"/>
       <c r="B25" s="49"/>
       <c r="C25" s="33"/>
@@ -2066,13 +2032,13 @@
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G25" s="58">
+      <c r="G25" s="53">
         <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H25" s="4"/>
     </row>
-    <row r="26" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="26" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2"/>
       <c r="B26" s="49"/>
       <c r="C26" s="33"/>
@@ -2082,13 +2048,13 @@
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G26" s="58">
+      <c r="G26" s="53">
         <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H26" s="4"/>
     </row>
-    <row r="27" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="27" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="2"/>
       <c r="B27" s="49"/>
       <c r="C27" s="33"/>
@@ -2098,13 +2064,13 @@
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G27" s="58">
+      <c r="G27" s="53">
         <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H27" s="4"/>
     </row>
-    <row r="28" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="28" spans="1:8" s="13" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="3"/>
       <c r="B28" s="50"/>
       <c r="C28" s="35"/>
@@ -2114,13 +2080,13 @@
         <f>SUM(ROUNDUP(Tabelle1[[#This Row],[Fahrzeit]]/5,0)*5, ROUNDUP(Tabelle1[[#This Row],[Direkter Fallkontakt]]/5,0)*5,ROUNDUP(Tabelle1[[#This Row],[Indirekte Fallbearbeitung]]/5,0)*5)</f>
         <v>0</v>
       </c>
-      <c r="G28" s="60">
+      <c r="G28" s="54">
         <f>Tabelle1[[#This Row],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H28" s="5"/>
     </row>
-    <row r="29" spans="1:8" s="13" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="29" spans="1:8" s="13" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="31"/>
       <c r="B29" s="46" t="s">
         <v>14</v>
@@ -2141,13 +2107,13 @@
         <f>SUBTOTAL(109,Tabelle1[Summe min])</f>
         <v>0</v>
       </c>
-      <c r="G29" s="61">
+      <c r="G29" s="55">
         <f>Tabelle1[[#Totals],[Summe min]]/1440</f>
         <v>0</v>
       </c>
       <c r="H29" s="32"/>
     </row>
-    <row r="30" spans="1:8" s="13" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="30" spans="1:8" s="13" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="40"/>
       <c r="B30" s="47" t="s">
         <v>15</v>
@@ -2162,7 +2128,7 @@
       <c r="G30" s="44"/>
       <c r="H30" s="10"/>
     </row>
-    <row r="31" spans="1:8" s="13" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="31" spans="1:8" s="13" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="41"/>
       <c r="B31" s="47" t="s">
         <v>16</v>
@@ -2185,7 +2151,7 @@
       </c>
       <c r="G31" s="45"/>
     </row>
-    <row r="32" spans="1:8" s="13" customFormat="1" ht="8.5" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="32" spans="1:8" s="13" customFormat="1" ht="8.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="41"/>
       <c r="B32" s="47"/>
       <c r="C32" s="43"/>
@@ -2194,7 +2160,7 @@
       <c r="F32" s="45"/>
       <c r="G32" s="45"/>
     </row>
-    <row r="33" spans="1:8" s="13" customFormat="1" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="33" spans="1:8" s="13" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A33" s="42"/>
       <c r="C33" s="48" t="str">
         <f>IF(OR(C31&lt;0,D31&lt;0,E31&lt;0),"Budget überzogen! Prüfen und genehmigen lassen.",IF(E29&gt;0.5*D29,"Zeiten für indirekte Fallbearbeitung überprüfen!",""))</f>
@@ -2205,7 +2171,7 @@
       <c r="F33" s="48"/>
       <c r="G33" s="48"/>
     </row>
-    <row r="34" spans="1:8" s="13" customFormat="1" ht="15.55" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="34" spans="1:8" s="13" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="11"/>
       <c r="B34" s="11"/>
       <c r="C34" s="11"/>
@@ -2216,32 +2182,31 @@
       <c r="H34" s="11"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="3QcLdSrvkVhIVnK36IghcSCivjGKP9GdF5KQ3ujOk9FBSupo+ya0i2e7/FsHCSqZSJZJ0mMUUpJAiNcTDq6o+A==" saltValue="IxK/hi5LX/tu/tCGlX+vLg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="4">
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A5:B5"/>
   </mergeCells>
-  <conditionalFormatting sqref="E29">
-    <cfRule type="expression" dxfId="4" priority="9">
-      <formula>E29&gt;0.5*D29</formula>
+  <conditionalFormatting sqref="C31:F31">
+    <cfRule type="expression" dxfId="4" priority="3">
+      <formula>C31&lt;0</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="4">
+      <formula>AND(C31&gt;=0,C31&lt;0.2*C30)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="5">
+      <formula>C31&gt;=0.2*C30</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C33:G33">
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>LEN($C$33)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C31:F31">
-    <cfRule type="expression" dxfId="2" priority="3">
-      <formula>C31&lt;0</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="4">
-      <formula>AND(C31&gt;=0,C31&lt;0.2*C30)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="5">
-      <formula>C31&gt;=0.2*C30</formula>
+  <conditionalFormatting sqref="E29">
+    <cfRule type="expression" dxfId="0" priority="9">
+      <formula>E29&gt;0.5*D29</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>

</xml_diff>